<commit_message>
Designer mock is ready
</commit_message>
<xml_diff>
--- a/trads/designer_translations.xlsx
+++ b/trads/designer_translations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28025"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Projects\outbreak-tools\misc\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/komlaviamevoin/Unsync-Working-Folders/outbreak-tools/trads/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CBCBFA52-0915-487F-BD37-D6142C88C192}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C13007D4-93A2-064E-B5E7-6D6CC6EF1936}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="43800" windowHeight="29960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LinelistTranslation" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2497" uniqueCount="2045">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2539" uniqueCount="2072">
   <si>
     <t>Tables for translations of the linelist</t>
   </si>
@@ -6169,13 +6169,94 @@
   </si>
   <si>
     <t>Saturday</t>
+  </si>
+  <si>
+    <t>btnFolderMulti</t>
+  </si>
+  <si>
+    <t>Load mutiple files/folders</t>
+  </si>
+  <si>
+    <t>Charger plusieurs fichiers/dossiers</t>
+  </si>
+  <si>
+    <t>تحميل ملفات/مجلدات متعددة</t>
+  </si>
+  <si>
+    <t>Cargar varios archivos/carpetas</t>
+  </si>
+  <si>
+    <t>Carregar vários ficheiros/pastas</t>
+  </si>
+  <si>
+    <t>btnAddMulti</t>
+  </si>
+  <si>
+    <t>btnResMulti</t>
+  </si>
+  <si>
+    <t>Resize</t>
+  </si>
+  <si>
+    <t>Supprimer des lignes</t>
+  </si>
+  <si>
+    <t>btnImpMulti</t>
+  </si>
+  <si>
+    <t>Import</t>
+  </si>
+  <si>
+    <t>Importer</t>
+  </si>
+  <si>
+    <t>btnExportMulti</t>
+  </si>
+  <si>
+    <t>Importação</t>
+  </si>
+  <si>
+    <t>Importar</t>
+  </si>
+  <si>
+    <t>يستورد</t>
+  </si>
+  <si>
+    <t>إضافة صفوف</t>
+  </si>
+  <si>
+    <t>تغيير الحجم</t>
+  </si>
+  <si>
+    <t>Cambiar el tamaño</t>
+  </si>
+  <si>
+    <t>Redimensionar</t>
+  </si>
+  <si>
+    <t>btnImpTrans</t>
+  </si>
+  <si>
+    <t>btnDupMulti</t>
+  </si>
+  <si>
+    <t>Duplicate</t>
+  </si>
+  <si>
+    <t>Dupliquer</t>
+  </si>
+  <si>
+    <t>Duplicada</t>
+  </si>
+  <si>
+    <t>ينسخ</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="9"/>
       <color rgb="FF000000"/>
@@ -6205,12 +6286,20 @@
       <sz val="9"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="9"/>
       <color theme="0"/>
       <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Helvetica"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -6290,7 +6379,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -6313,6 +6402,7 @@
     <xf numFmtId="0" fontId="4" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -6671,8 +6761,8 @@
 </file>
 
 <file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="t_tradmsg" displayName="t_tradmsg" ref="B6:G72" totalsRowShown="0">
-  <autoFilter ref="B6:G72" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{00000000-000C-0000-FFFF-FFFF04000000}" name="t_tradmsg" displayName="t_tradmsg" ref="B6:G79" totalsRowShown="0">
+  <autoFilter ref="B6:G79" xr:uid="{00000000-0009-0000-0100-000007000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="B7:G72">
     <sortCondition ref="C6:C72"/>
   </sortState>
@@ -6689,8 +6779,8 @@
 </file>
 
 <file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="t_tradrange" displayName="t_tradrange" ref="B76:G90" totalsRowShown="0">
-  <autoFilter ref="B76:G90" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{00000000-000C-0000-FFFF-FFFF05000000}" name="t_tradrange" displayName="t_tradrange" ref="B83:G97" totalsRowShown="0">
+  <autoFilter ref="B83:G97" xr:uid="{00000000-0009-0000-0100-000008000000}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0500-000001000000}" name="MSG_ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0500-000002000000}" name="ENG"/>
@@ -6704,8 +6794,8 @@
 </file>
 
 <file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="t_tradshape" displayName="t_tradshape" ref="B94:G107" totalsRowShown="0">
-  <autoFilter ref="B94:G107" xr:uid="{00000000-0009-0000-0100-000009000000}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{00000000-000C-0000-FFFF-FFFF06000000}" name="t_tradshape" displayName="t_tradshape" ref="B101:G114" totalsRowShown="0">
+  <autoFilter ref="B101:G114" xr:uid="{00000000-0009-0000-0100-000009000000}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0600-000001000000}" name="MSG_ID"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0600-000002000000}" name="ENG"/>
@@ -6719,8 +6809,8 @@
 </file>
 
 <file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CBF201D7-64ED-443F-AE13-88E0A1D19EA7}" name="t_traddrop" displayName="t_traddrop" ref="B113:G114" totalsRowShown="0" headerRowDxfId="10" dataDxfId="8" headerRowBorderDxfId="9" tableBorderDxfId="7" totalsRowBorderDxfId="6">
-  <autoFilter ref="B113:G114" xr:uid="{CBF201D7-64ED-443F-AE13-88E0A1D19EA7}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{CBF201D7-64ED-443F-AE13-88E0A1D19EA7}" name="t_traddrop" displayName="t_traddrop" ref="B120:G121" totalsRowShown="0" headerRowDxfId="10" dataDxfId="8" headerRowBorderDxfId="9" tableBorderDxfId="7" totalsRowBorderDxfId="6">
+  <autoFilter ref="B120:G121" xr:uid="{CBF201D7-64ED-443F-AE13-88E0A1D19EA7}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{017F9F65-DA3E-4D2D-A8A9-86B0311704B8}" name="MSG_ID" dataDxfId="5"/>
     <tableColumn id="2" xr3:uid="{8CB7068D-F258-480F-84FF-DA8083B35313}" name="ENG" dataDxfId="4"/>
@@ -7014,12 +7104,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="B2:G334"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="200" width="35.6640625" customWidth="1"/>
+    <col min="1" max="200" width="35.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -7029,7 +7119,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -7037,7 +7127,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B4" s="3" t="s">
         <v>2</v>
       </c>
@@ -7047,7 +7137,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -7055,7 +7145,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
@@ -7075,7 +7165,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B7" s="2" t="s">
         <v>9</v>
       </c>
@@ -7095,7 +7185,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B8" s="2" t="s">
         <v>15</v>
       </c>
@@ -7115,7 +7205,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B9" s="2" t="s">
         <v>21</v>
       </c>
@@ -7135,7 +7225,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B10" s="2" t="s">
         <v>27</v>
       </c>
@@ -7155,7 +7245,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B11" s="2" t="s">
         <v>33</v>
       </c>
@@ -7175,7 +7265,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B12" s="2" t="s">
         <v>37</v>
       </c>
@@ -7195,7 +7285,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B13" s="2" t="s">
         <v>42</v>
       </c>
@@ -7215,7 +7305,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B14" s="2" t="s">
         <v>45</v>
       </c>
@@ -7235,7 +7325,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B15" s="2" t="s">
         <v>50</v>
       </c>
@@ -7255,7 +7345,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="16" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B16" s="2" t="s">
         <v>56</v>
       </c>
@@ -7275,7 +7365,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B19" s="3" t="s">
         <v>62</v>
       </c>
@@ -7285,7 +7375,7 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
     </row>
-    <row r="20" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -7293,7 +7383,7 @@
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
     </row>
-    <row r="21" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B21" s="2" t="s">
         <v>3</v>
       </c>
@@ -7313,7 +7403,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B22" s="2" t="s">
         <v>2013</v>
       </c>
@@ -7333,7 +7423,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="23" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B23" s="2" t="s">
         <v>2019</v>
       </c>
@@ -7353,7 +7443,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="24" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B24" s="2" t="s">
         <v>63</v>
       </c>
@@ -7373,7 +7463,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B25" s="2" t="s">
         <v>67</v>
       </c>
@@ -7393,7 +7483,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="26" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B26" s="2" t="s">
         <v>73</v>
       </c>
@@ -7413,7 +7503,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B27" s="2" t="s">
         <v>79</v>
       </c>
@@ -7433,7 +7523,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B28" s="2" t="s">
         <v>85</v>
       </c>
@@ -7453,7 +7543,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="29" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B29" s="2" t="s">
         <v>91</v>
       </c>
@@ -7473,7 +7563,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B30" s="2" t="s">
         <v>97</v>
       </c>
@@ -7493,7 +7583,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="31" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B31" s="2" t="s">
         <v>103</v>
       </c>
@@ -7513,7 +7603,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="32" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B32" s="2" t="s">
         <v>108</v>
       </c>
@@ -7533,7 +7623,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="33" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B33" s="2" t="s">
         <v>113</v>
       </c>
@@ -7553,7 +7643,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="34" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B34" s="2" t="s">
         <v>118</v>
       </c>
@@ -7573,7 +7663,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="35" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B35" s="2" t="s">
         <v>123</v>
       </c>
@@ -7593,7 +7683,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="36" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B36" s="2" t="s">
         <v>129</v>
       </c>
@@ -7613,7 +7703,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="37" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B37" s="2" t="s">
         <v>135</v>
       </c>
@@ -7633,7 +7723,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="38" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B38" s="2" t="s">
         <v>140</v>
       </c>
@@ -7653,7 +7743,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="39" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B39" s="2" t="s">
         <v>145</v>
       </c>
@@ -7673,7 +7763,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="40" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B40" s="2" t="s">
         <v>150</v>
       </c>
@@ -7693,7 +7783,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="41" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B41" s="2" t="s">
         <v>156</v>
       </c>
@@ -7713,7 +7803,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="42" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B42" s="2" t="s">
         <v>161</v>
       </c>
@@ -7733,7 +7823,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="43" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B43" s="2" t="s">
         <v>166</v>
       </c>
@@ -7753,7 +7843,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="44" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B44" s="2" t="s">
         <v>172</v>
       </c>
@@ -7773,7 +7863,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="45" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B45" s="2" t="s">
         <v>178</v>
       </c>
@@ -7793,7 +7883,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="46" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B46" s="2" t="s">
         <v>183</v>
       </c>
@@ -7813,7 +7903,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="47" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B47" s="2" t="s">
         <v>189</v>
       </c>
@@ -7833,7 +7923,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="48" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B48" s="2" t="s">
         <v>195</v>
       </c>
@@ -7853,7 +7943,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="49" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B49" s="2" t="s">
         <v>201</v>
       </c>
@@ -7873,7 +7963,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="50" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B50" s="2" t="s">
         <v>207</v>
       </c>
@@ -7893,7 +7983,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="51" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B51" s="2" t="s">
         <v>212</v>
       </c>
@@ -7913,7 +8003,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="52" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B52" s="2" t="s">
         <v>217</v>
       </c>
@@ -7933,7 +8023,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="53" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B53" s="2" t="s">
         <v>222</v>
       </c>
@@ -7953,7 +8043,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="54" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B54" s="2" t="s">
         <v>228</v>
       </c>
@@ -7973,7 +8063,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="55" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B55" s="2" t="s">
         <v>230</v>
       </c>
@@ -7993,7 +8083,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="56" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B56" s="2" t="s">
         <v>235</v>
       </c>
@@ -8013,7 +8103,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B57" s="2" t="s">
         <v>240</v>
       </c>
@@ -8033,7 +8123,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="58" spans="2:7" ht="36" x14ac:dyDescent="0.2">
+    <row r="58" spans="2:7" ht="39" x14ac:dyDescent="0.15">
       <c r="B58" s="2" t="s">
         <v>245</v>
       </c>
@@ -8053,7 +8143,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="59" spans="2:7" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="2:7" ht="51" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B59" s="4" t="s">
         <v>2007</v>
       </c>
@@ -8073,7 +8163,7 @@
         <v>2012</v>
       </c>
     </row>
-    <row r="60" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B60" s="2" t="s">
         <v>250</v>
       </c>
@@ -8093,7 +8183,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="61" spans="2:7" ht="60" x14ac:dyDescent="0.2">
+    <row r="61" spans="2:7" ht="52" x14ac:dyDescent="0.15">
       <c r="B61" s="2" t="s">
         <v>256</v>
       </c>
@@ -8113,7 +8203,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="62" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B62" s="2" t="s">
         <v>262</v>
       </c>
@@ -8133,7 +8223,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="63" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B63" s="2" t="s">
         <v>268</v>
       </c>
@@ -8153,7 +8243,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="64" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B64" s="2" t="s">
         <v>274</v>
       </c>
@@ -8173,7 +8263,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="65" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B65" s="2" t="s">
         <v>279</v>
       </c>
@@ -8193,7 +8283,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="66" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B66" s="2" t="s">
         <v>285</v>
       </c>
@@ -8211,7 +8301,7 @@
       </c>
       <c r="G66" s="2"/>
     </row>
-    <row r="67" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B67" s="2" t="s">
         <v>289</v>
       </c>
@@ -8231,7 +8321,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="68" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B68" s="2" t="s">
         <v>294</v>
       </c>
@@ -8251,7 +8341,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="69" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B69" s="2" t="s">
         <v>300</v>
       </c>
@@ -8271,7 +8361,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="70" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B70" s="2" t="s">
         <v>305</v>
       </c>
@@ -8291,7 +8381,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="71" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B71" s="2" t="s">
         <v>310</v>
       </c>
@@ -8311,7 +8401,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="72" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B72" s="2" t="s">
         <v>316</v>
       </c>
@@ -8331,7 +8421,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="73" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B73" s="2" t="s">
         <v>322</v>
       </c>
@@ -8351,7 +8441,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="74" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B74" s="2" t="s">
         <v>328</v>
       </c>
@@ -8371,7 +8461,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="75" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B75" s="2" t="s">
         <v>334</v>
       </c>
@@ -8391,7 +8481,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="76" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="76" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B76" s="2" t="s">
         <v>340</v>
       </c>
@@ -8411,7 +8501,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="77" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B77" s="2" t="s">
         <v>346</v>
       </c>
@@ -8431,7 +8521,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="78" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B78" s="2" t="s">
         <v>352</v>
       </c>
@@ -8451,7 +8541,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="79" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B79" s="2" t="s">
         <v>357</v>
       </c>
@@ -8471,7 +8561,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="80" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="80" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B80" s="2" t="s">
         <v>362</v>
       </c>
@@ -8491,7 +8581,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="81" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="81" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B81" s="2" t="s">
         <v>368</v>
       </c>
@@ -8511,7 +8601,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="82" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="82" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B82" s="2" t="s">
         <v>373</v>
       </c>
@@ -8531,7 +8621,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="83" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="83" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B83" s="2" t="s">
         <v>378</v>
       </c>
@@ -8551,7 +8641,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="84" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="84" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B84" s="2" t="s">
         <v>384</v>
       </c>
@@ -8571,7 +8661,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="85" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="85" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B85" s="2" t="s">
         <v>389</v>
       </c>
@@ -8591,7 +8681,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="86" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="86" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B86" s="2" t="s">
         <v>394</v>
       </c>
@@ -8611,7 +8701,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="87" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="87" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B87" s="2" t="s">
         <v>399</v>
       </c>
@@ -8631,7 +8721,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="88" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="88" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B88" s="2" t="s">
         <v>405</v>
       </c>
@@ -8651,7 +8741,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="89" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="89" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B89" s="2" t="s">
         <v>410</v>
       </c>
@@ -8671,7 +8761,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="90" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="90" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B90" s="2" t="s">
         <v>416</v>
       </c>
@@ -8691,7 +8781,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="91" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="91" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B91" s="2" t="s">
         <v>421</v>
       </c>
@@ -8711,7 +8801,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="92" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="92" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B92" s="2" t="s">
         <v>427</v>
       </c>
@@ -8731,7 +8821,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="93" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="93" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B93" s="2" t="s">
         <v>433</v>
       </c>
@@ -8751,7 +8841,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="94" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="94" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B94" s="2" t="s">
         <v>438</v>
       </c>
@@ -8771,7 +8861,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="95" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="95" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B95" s="2" t="s">
         <v>444</v>
       </c>
@@ -8791,7 +8881,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="96" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="96" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B96" s="2" t="s">
         <v>449</v>
       </c>
@@ -8811,7 +8901,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="97" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="97" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B97" s="2" t="s">
         <v>453</v>
       </c>
@@ -8831,7 +8921,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="98" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="98" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B98" s="2" t="s">
         <v>459</v>
       </c>
@@ -8851,7 +8941,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="99" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="99" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B99" s="2" t="s">
         <v>465</v>
       </c>
@@ -8871,7 +8961,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="100" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="100" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B100" s="2" t="s">
         <v>471</v>
       </c>
@@ -8891,7 +8981,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="101" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="101" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B101" s="2" t="s">
         <v>477</v>
       </c>
@@ -8911,7 +9001,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="102" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="102" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B102" s="2" t="s">
         <v>483</v>
       </c>
@@ -8931,7 +9021,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="103" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="103" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B103" s="2" t="s">
         <v>489</v>
       </c>
@@ -8951,7 +9041,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="104" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="104" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B104" s="2" t="s">
         <v>494</v>
       </c>
@@ -8971,7 +9061,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="105" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="105" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B105" s="2" t="s">
         <v>500</v>
       </c>
@@ -8991,7 +9081,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="106" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="106" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B106" s="2" t="s">
         <v>506</v>
       </c>
@@ -9011,7 +9101,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="107" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="107" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B107" s="2" t="s">
         <v>511</v>
       </c>
@@ -9031,7 +9121,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="108" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="108" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B108" s="2" t="s">
         <v>517</v>
       </c>
@@ -9051,7 +9141,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="109" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="109" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B109" s="2" t="s">
         <v>523</v>
       </c>
@@ -9071,7 +9161,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="110" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="110" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B110" s="2" t="s">
         <v>528</v>
       </c>
@@ -9091,7 +9181,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="111" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="111" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B111" s="2" t="s">
         <v>534</v>
       </c>
@@ -9111,7 +9201,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="112" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="112" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B112" s="2" t="s">
         <v>540</v>
       </c>
@@ -9131,7 +9221,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="113" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="113" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B113" s="2" t="s">
         <v>546</v>
       </c>
@@ -9151,7 +9241,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="114" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="114" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B114" s="2" t="s">
         <v>552</v>
       </c>
@@ -9171,7 +9261,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="115" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="115" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B115" s="2" t="s">
         <v>558</v>
       </c>
@@ -9191,7 +9281,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="116" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="116" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B116" s="2" t="s">
         <v>563</v>
       </c>
@@ -9211,7 +9301,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="117" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="117" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B117" s="2" t="s">
         <v>569</v>
       </c>
@@ -9231,7 +9321,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="118" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="118" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B118" s="2" t="s">
         <v>573</v>
       </c>
@@ -9251,7 +9341,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="119" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="119" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B119" s="2" t="s">
         <v>579</v>
       </c>
@@ -9271,7 +9361,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="120" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="120" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B120" s="2" t="s">
         <v>585</v>
       </c>
@@ -9291,7 +9381,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="121" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="121" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B121" s="2" t="s">
         <v>591</v>
       </c>
@@ -9311,7 +9401,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="122" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="122" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B122" s="2" t="s">
         <v>597</v>
       </c>
@@ -9331,7 +9421,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="123" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="123" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B123" s="2" t="s">
         <v>603</v>
       </c>
@@ -9351,7 +9441,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="124" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="124" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B124" s="2" t="s">
         <v>609</v>
       </c>
@@ -9371,7 +9461,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="125" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="125" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B125" s="2" t="s">
         <v>615</v>
       </c>
@@ -9391,7 +9481,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="126" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="126" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B126" s="2" t="s">
         <v>621</v>
       </c>
@@ -9411,7 +9501,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="127" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="127" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B127" s="2" t="s">
         <v>627</v>
       </c>
@@ -9431,7 +9521,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="128" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="128" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B128" s="2" t="s">
         <v>633</v>
       </c>
@@ -9451,7 +9541,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="129" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="129" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B129" s="2" t="s">
         <v>639</v>
       </c>
@@ -9471,7 +9561,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="130" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="130" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B130" s="2" t="s">
         <v>645</v>
       </c>
@@ -9491,7 +9581,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="131" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="131" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B131" s="2" t="s">
         <v>650</v>
       </c>
@@ -9511,7 +9601,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="132" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="132" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B132" s="2" t="s">
         <v>655</v>
       </c>
@@ -9531,7 +9621,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="133" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="133" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B133" s="2" t="s">
         <v>660</v>
       </c>
@@ -9551,7 +9641,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="134" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="134" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B134" s="2" t="s">
         <v>665</v>
       </c>
@@ -9571,7 +9661,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="135" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="135" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B135" s="2" t="s">
         <v>671</v>
       </c>
@@ -9591,7 +9681,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="136" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="136" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B136" s="2" t="s">
         <v>676</v>
       </c>
@@ -9611,7 +9701,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="137" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="137" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B137" s="2" t="s">
         <v>681</v>
       </c>
@@ -9631,7 +9721,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="138" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="138" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B138" s="2" t="s">
         <v>686</v>
       </c>
@@ -9651,7 +9741,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="139" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="139" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B139" s="2" t="s">
         <v>689</v>
       </c>
@@ -9671,7 +9761,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="140" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="140" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B140" s="2" t="s">
         <v>694</v>
       </c>
@@ -9691,7 +9781,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="141" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="141" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B141" s="2" t="s">
         <v>700</v>
       </c>
@@ -9711,7 +9801,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="142" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="142" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B142" s="2" t="s">
         <v>705</v>
       </c>
@@ -9729,7 +9819,7 @@
       </c>
       <c r="G142" s="2"/>
     </row>
-    <row r="143" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="143" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B143" s="2" t="s">
         <v>710</v>
       </c>
@@ -9749,7 +9839,7 @@
         <v>715</v>
       </c>
     </row>
-    <row r="144" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="144" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B144" s="2" t="s">
         <v>716</v>
       </c>
@@ -9769,7 +9859,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="145" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="145" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B145" s="2" t="s">
         <v>722</v>
       </c>
@@ -9789,7 +9879,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="146" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="146" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B146" s="2" t="s">
         <v>725</v>
       </c>
@@ -9809,7 +9899,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="147" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="147" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B147" s="2" t="s">
         <v>730</v>
       </c>
@@ -9829,7 +9919,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="148" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="148" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B148" s="2" t="s">
         <v>735</v>
       </c>
@@ -9849,7 +9939,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="149" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="149" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B149" s="2" t="s">
         <v>741</v>
       </c>
@@ -9867,7 +9957,7 @@
       </c>
       <c r="G149" s="2"/>
     </row>
-    <row r="150" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="150" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B150" s="2" t="s">
         <v>746</v>
       </c>
@@ -9887,7 +9977,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="151" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="151" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B151" s="2" t="s">
         <v>752</v>
       </c>
@@ -9907,7 +9997,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="152" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="152" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B152" s="2" t="s">
         <v>758</v>
       </c>
@@ -9927,7 +10017,7 @@
         <v>763</v>
       </c>
     </row>
-    <row r="153" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="153" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B153" s="2" t="s">
         <v>764</v>
       </c>
@@ -9947,7 +10037,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="154" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="154" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B154" s="2" t="s">
         <v>767</v>
       </c>
@@ -9967,7 +10057,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="155" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="155" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B155" s="2" t="s">
         <v>773</v>
       </c>
@@ -9987,7 +10077,7 @@
         <v>778</v>
       </c>
     </row>
-    <row r="156" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="156" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B156" s="2" t="s">
         <v>779</v>
       </c>
@@ -10007,7 +10097,7 @@
         <v>784</v>
       </c>
     </row>
-    <row r="157" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="157" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B157" s="2" t="s">
         <v>785</v>
       </c>
@@ -10027,7 +10117,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="158" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="158" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B158" s="2" t="s">
         <v>786</v>
       </c>
@@ -10047,7 +10137,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="159" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="159" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B159" s="2" t="s">
         <v>792</v>
       </c>
@@ -10067,7 +10157,7 @@
         <v>797</v>
       </c>
     </row>
-    <row r="160" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="160" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B160" s="2" t="s">
         <v>798</v>
       </c>
@@ -10087,7 +10177,7 @@
         <v>803</v>
       </c>
     </row>
-    <row r="161" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="161" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B161" s="2" t="s">
         <v>804</v>
       </c>
@@ -10107,7 +10197,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="162" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="162" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B162" s="2" t="s">
         <v>809</v>
       </c>
@@ -10127,7 +10217,7 @@
         <v>814</v>
       </c>
     </row>
-    <row r="163" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="163" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B163" s="2" t="s">
         <v>815</v>
       </c>
@@ -10147,7 +10237,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="164" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="164" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B164" s="2" t="s">
         <v>821</v>
       </c>
@@ -10167,7 +10257,7 @@
         <v>823</v>
       </c>
     </row>
-    <row r="165" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="165" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B165" s="2" t="s">
         <v>824</v>
       </c>
@@ -10187,7 +10277,7 @@
         <v>829</v>
       </c>
     </row>
-    <row r="166" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="166" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B166" s="2" t="s">
         <v>830</v>
       </c>
@@ -10207,7 +10297,7 @@
         <v>835</v>
       </c>
     </row>
-    <row r="167" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="167" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B167" s="2" t="s">
         <v>836</v>
       </c>
@@ -10227,7 +10317,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="168" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="168" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B168" s="2" t="s">
         <v>841</v>
       </c>
@@ -10247,7 +10337,7 @@
         <v>845</v>
       </c>
     </row>
-    <row r="169" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="169" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B169" s="2" t="s">
         <v>846</v>
       </c>
@@ -10267,7 +10357,7 @@
         <v>851</v>
       </c>
     </row>
-    <row r="170" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="170" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B170" s="2" t="s">
         <v>852</v>
       </c>
@@ -10287,7 +10377,7 @@
         <v>856</v>
       </c>
     </row>
-    <row r="171" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="171" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B171" s="2" t="s">
         <v>857</v>
       </c>
@@ -10307,7 +10397,7 @@
         <v>858</v>
       </c>
     </row>
-    <row r="172" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="172" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B172" s="2" t="s">
         <v>862</v>
       </c>
@@ -10327,7 +10417,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="173" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="173" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B173" s="2" t="s">
         <v>868</v>
       </c>
@@ -10347,7 +10437,7 @@
         <v>873</v>
       </c>
     </row>
-    <row r="174" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="174" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B174" s="2" t="s">
         <v>874</v>
       </c>
@@ -10367,7 +10457,7 @@
         <v>879</v>
       </c>
     </row>
-    <row r="175" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="175" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B175" s="2" t="s">
         <v>880</v>
       </c>
@@ -10387,7 +10477,7 @@
         <v>885</v>
       </c>
     </row>
-    <row r="176" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="176" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B176" s="2" t="s">
         <v>886</v>
       </c>
@@ -10407,7 +10497,7 @@
         <v>890</v>
       </c>
     </row>
-    <row r="177" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="177" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B177" s="2" t="s">
         <v>1991</v>
       </c>
@@ -10427,7 +10517,7 @@
         <v>1996</v>
       </c>
     </row>
-    <row r="178" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="178" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B178" s="4" t="s">
         <v>1997</v>
       </c>
@@ -10447,7 +10537,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="181" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="181" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B181" s="3" t="s">
         <v>891</v>
       </c>
@@ -10457,7 +10547,7 @@
       <c r="F181" s="2"/>
       <c r="G181" s="2"/>
     </row>
-    <row r="182" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="182" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B182" s="2"/>
       <c r="C182" s="2"/>
       <c r="D182" s="2"/>
@@ -10465,7 +10555,7 @@
       <c r="F182" s="2"/>
       <c r="G182" s="2"/>
     </row>
-    <row r="183" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="183" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B183" s="2" t="s">
         <v>3</v>
       </c>
@@ -10485,7 +10575,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="184" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="184" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B184" s="2" t="s">
         <v>892</v>
       </c>
@@ -10505,7 +10595,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="185" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="185" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B185" s="2" t="s">
         <v>898</v>
       </c>
@@ -10525,7 +10615,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="186" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="186" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B186" s="2" t="s">
         <v>901</v>
       </c>
@@ -10545,7 +10635,7 @@
         <v>906</v>
       </c>
     </row>
-    <row r="187" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="187" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B187" s="2" t="s">
         <v>907</v>
       </c>
@@ -10565,7 +10655,7 @@
         <v>910</v>
       </c>
     </row>
-    <row r="188" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="188" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B188" s="2" t="s">
         <v>911</v>
       </c>
@@ -10585,7 +10675,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="189" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="189" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B189" s="2" t="s">
         <v>917</v>
       </c>
@@ -10605,7 +10695,7 @@
         <v>922</v>
       </c>
     </row>
-    <row r="190" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="190" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B190" s="2" t="s">
         <v>923</v>
       </c>
@@ -10625,7 +10715,7 @@
         <v>927</v>
       </c>
     </row>
-    <row r="191" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="191" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B191" s="2" t="s">
         <v>928</v>
       </c>
@@ -10645,7 +10735,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="192" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="192" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B192" s="2" t="s">
         <v>934</v>
       </c>
@@ -10665,7 +10755,7 @@
         <v>939</v>
       </c>
     </row>
-    <row r="193" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="193" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B193" s="2" t="s">
         <v>940</v>
       </c>
@@ -10685,7 +10775,7 @@
         <v>945</v>
       </c>
     </row>
-    <row r="194" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="194" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B194" s="2" t="s">
         <v>946</v>
       </c>
@@ -10705,7 +10795,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="195" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="195" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B195" s="2" t="s">
         <v>948</v>
       </c>
@@ -10725,7 +10815,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="196" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="196" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B196" s="2" t="s">
         <v>954</v>
       </c>
@@ -10745,7 +10835,7 @@
         <v>959</v>
       </c>
     </row>
-    <row r="197" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="197" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B197" s="2" t="s">
         <v>960</v>
       </c>
@@ -10765,7 +10855,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="198" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="198" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B198" s="2" t="s">
         <v>965</v>
       </c>
@@ -10785,7 +10875,7 @@
         <v>969</v>
       </c>
     </row>
-    <row r="199" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="199" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B199" s="2" t="s">
         <v>970</v>
       </c>
@@ -10805,7 +10895,7 @@
         <v>971</v>
       </c>
     </row>
-    <row r="200" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="200" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B200" s="2" t="s">
         <v>972</v>
       </c>
@@ -10825,7 +10915,7 @@
         <v>976</v>
       </c>
     </row>
-    <row r="201" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="201" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B201" s="2" t="s">
         <v>977</v>
       </c>
@@ -10845,7 +10935,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="202" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="202" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B202" s="2" t="s">
         <v>982</v>
       </c>
@@ -10865,7 +10955,7 @@
         <v>985</v>
       </c>
     </row>
-    <row r="203" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="203" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B203" s="2" t="s">
         <v>986</v>
       </c>
@@ -10885,7 +10975,7 @@
         <v>990</v>
       </c>
     </row>
-    <row r="204" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="204" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B204" s="2" t="s">
         <v>991</v>
       </c>
@@ -10905,7 +10995,7 @@
         <v>992</v>
       </c>
     </row>
-    <row r="205" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="205" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B205" s="2" t="s">
         <v>993</v>
       </c>
@@ -10925,7 +11015,7 @@
         <v>994</v>
       </c>
     </row>
-    <row r="206" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="206" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B206" s="2" t="s">
         <v>995</v>
       </c>
@@ -10945,7 +11035,7 @@
         <v>996</v>
       </c>
     </row>
-    <row r="207" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="207" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B207" s="2" t="s">
         <v>997</v>
       </c>
@@ -10965,7 +11055,7 @@
         <v>998</v>
       </c>
     </row>
-    <row r="208" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="208" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B208" s="2" t="s">
         <v>999</v>
       </c>
@@ -10985,7 +11075,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="209" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="209" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B209" s="2" t="s">
         <v>1004</v>
       </c>
@@ -11005,7 +11095,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="210" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="210" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B210" s="2" t="s">
         <v>1006</v>
       </c>
@@ -11025,7 +11115,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="211" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="211" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B211" s="2" t="s">
         <v>1007</v>
       </c>
@@ -11045,7 +11135,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="212" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="212" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B212" s="2" t="s">
         <v>1013</v>
       </c>
@@ -11065,7 +11155,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="213" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="213" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B213" s="2" t="s">
         <v>1014</v>
       </c>
@@ -11085,7 +11175,7 @@
         <v>1019</v>
       </c>
     </row>
-    <row r="214" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="214" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B214" s="2" t="s">
         <v>1020</v>
       </c>
@@ -11105,7 +11195,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="215" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="215" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B215" s="2" t="s">
         <v>1025</v>
       </c>
@@ -11125,7 +11215,7 @@
         <v>1030</v>
       </c>
     </row>
-    <row r="216" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="216" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B216" s="2" t="s">
         <v>1031</v>
       </c>
@@ -11145,7 +11235,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="217" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="217" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B217" s="2" t="s">
         <v>1032</v>
       </c>
@@ -11165,7 +11255,7 @@
         <v>1037</v>
       </c>
     </row>
-    <row r="218" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="218" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B218" s="2" t="s">
         <v>1038</v>
       </c>
@@ -11185,7 +11275,7 @@
         <v>1043</v>
       </c>
     </row>
-    <row r="219" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="219" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B219" s="2" t="s">
         <v>1044</v>
       </c>
@@ -11205,7 +11295,7 @@
         <v>1049</v>
       </c>
     </row>
-    <row r="220" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="220" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B220" s="2" t="s">
         <v>1050</v>
       </c>
@@ -11225,7 +11315,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="221" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="221" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B221" s="2" t="s">
         <v>1051</v>
       </c>
@@ -11245,7 +11335,7 @@
         <v>1056</v>
       </c>
     </row>
-    <row r="222" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="222" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B222" s="2" t="s">
         <v>1057</v>
       </c>
@@ -11265,7 +11355,7 @@
         <v>1062</v>
       </c>
     </row>
-    <row r="223" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="223" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B223" s="2" t="s">
         <v>1063</v>
       </c>
@@ -11285,7 +11375,7 @@
         <v>1068</v>
       </c>
     </row>
-    <row r="224" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="224" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B224" s="2" t="s">
         <v>1069</v>
       </c>
@@ -11305,7 +11395,7 @@
         <v>1074</v>
       </c>
     </row>
-    <row r="225" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="225" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B225" s="2" t="s">
         <v>1075</v>
       </c>
@@ -11325,7 +11415,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="226" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="226" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B226" s="2" t="s">
         <v>1076</v>
       </c>
@@ -11345,7 +11435,7 @@
         <v>1080</v>
       </c>
     </row>
-    <row r="227" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="227" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B227" s="2" t="s">
         <v>1081</v>
       </c>
@@ -11365,7 +11455,7 @@
         <v>1086</v>
       </c>
     </row>
-    <row r="228" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="228" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B228" s="2" t="s">
         <v>1087</v>
       </c>
@@ -11385,7 +11475,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="229" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="229" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B229" s="2" t="s">
         <v>1091</v>
       </c>
@@ -11405,7 +11495,7 @@
         <v>1096</v>
       </c>
     </row>
-    <row r="230" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="230" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B230" s="2" t="s">
         <v>1097</v>
       </c>
@@ -11425,7 +11515,7 @@
         <v>939</v>
       </c>
     </row>
-    <row r="231" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="231" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B231" s="2" t="s">
         <v>1098</v>
       </c>
@@ -11445,7 +11535,7 @@
         <v>945</v>
       </c>
     </row>
-    <row r="232" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="232" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B232" s="2" t="s">
         <v>1102</v>
       </c>
@@ -11465,7 +11555,7 @@
         <v>1107</v>
       </c>
     </row>
-    <row r="233" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="233" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B233" s="2" t="s">
         <v>1108</v>
       </c>
@@ -11485,7 +11575,7 @@
         <v>1989</v>
       </c>
     </row>
-    <row r="234" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="234" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B234" s="2" t="s">
         <v>1109</v>
       </c>
@@ -11505,7 +11595,7 @@
         <v>1110</v>
       </c>
     </row>
-    <row r="235" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="235" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B235" s="2" t="s">
         <v>1113</v>
       </c>
@@ -11525,7 +11615,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="236" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="236" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B236" s="2" t="s">
         <v>1114</v>
       </c>
@@ -11545,7 +11635,7 @@
         <v>1118</v>
       </c>
     </row>
-    <row r="237" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="237" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B237" s="2" t="s">
         <v>1119</v>
       </c>
@@ -11565,7 +11655,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="238" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="238" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B238" s="2" t="s">
         <v>1120</v>
       </c>
@@ -11585,7 +11675,7 @@
         <v>1125</v>
       </c>
     </row>
-    <row r="239" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="239" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B239" s="2" t="s">
         <v>1126</v>
       </c>
@@ -11605,7 +11695,7 @@
         <v>1131</v>
       </c>
     </row>
-    <row r="240" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="240" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B240" s="2" t="s">
         <v>1132</v>
       </c>
@@ -11625,7 +11715,7 @@
         <v>1131</v>
       </c>
     </row>
-    <row r="241" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="241" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B241" s="2" t="s">
         <v>1133</v>
       </c>
@@ -11645,7 +11735,7 @@
         <v>1138</v>
       </c>
     </row>
-    <row r="242" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="242" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B242" s="2" t="s">
         <v>1139</v>
       </c>
@@ -11665,7 +11755,7 @@
         <v>1141</v>
       </c>
     </row>
-    <row r="243" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="243" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B243" s="2" t="s">
         <v>1142</v>
       </c>
@@ -11685,7 +11775,7 @@
         <v>1141</v>
       </c>
     </row>
-    <row r="244" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="244" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B244" s="2" t="s">
         <v>1143</v>
       </c>
@@ -11705,7 +11795,7 @@
         <v>1145</v>
       </c>
     </row>
-    <row r="245" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="245" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B245" s="2" t="s">
         <v>1146</v>
       </c>
@@ -11725,7 +11815,7 @@
         <v>1145</v>
       </c>
     </row>
-    <row r="246" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="246" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B246" s="2" t="s">
         <v>1147</v>
       </c>
@@ -11745,7 +11835,7 @@
         <v>1149</v>
       </c>
     </row>
-    <row r="247" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="247" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B247" s="2" t="s">
         <v>1150</v>
       </c>
@@ -11765,7 +11855,7 @@
         <v>1149</v>
       </c>
     </row>
-    <row r="248" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="248" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B248" s="2" t="s">
         <v>1151</v>
       </c>
@@ -11785,7 +11875,7 @@
         <v>1153</v>
       </c>
     </row>
-    <row r="249" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="249" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B249" s="2" t="s">
         <v>1154</v>
       </c>
@@ -11805,7 +11895,7 @@
         <v>1153</v>
       </c>
     </row>
-    <row r="250" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="250" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B250" s="2" t="s">
         <v>1155</v>
       </c>
@@ -11825,7 +11915,7 @@
         <v>1160</v>
       </c>
     </row>
-    <row r="251" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="251" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B251" s="2" t="s">
         <v>1161</v>
       </c>
@@ -11845,7 +11935,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="252" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="252" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B252" s="2" t="s">
         <v>1164</v>
       </c>
@@ -11865,7 +11955,7 @@
         <v>1169</v>
       </c>
     </row>
-    <row r="253" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="253" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B253" s="2" t="s">
         <v>1170</v>
       </c>
@@ -11885,7 +11975,7 @@
         <v>1175</v>
       </c>
     </row>
-    <row r="254" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="254" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B254" s="2" t="s">
         <v>1176</v>
       </c>
@@ -11905,7 +11995,7 @@
         <v>1181</v>
       </c>
     </row>
-    <row r="255" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="255" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B255" s="2" t="s">
         <v>1182</v>
       </c>
@@ -11925,7 +12015,7 @@
         <v>1185</v>
       </c>
     </row>
-    <row r="256" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="256" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B256" s="2" t="s">
         <v>1186</v>
       </c>
@@ -11945,7 +12035,7 @@
         <v>1191</v>
       </c>
     </row>
-    <row r="257" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="257" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B257" s="2" t="s">
         <v>1192</v>
       </c>
@@ -11965,7 +12055,7 @@
         <v>1197</v>
       </c>
     </row>
-    <row r="258" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="258" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B258" s="2" t="s">
         <v>1198</v>
       </c>
@@ -11985,7 +12075,7 @@
         <v>1197</v>
       </c>
     </row>
-    <row r="259" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="259" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B259" s="2" t="s">
         <v>1199</v>
       </c>
@@ -12005,7 +12095,7 @@
         <v>1204</v>
       </c>
     </row>
-    <row r="260" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="260" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B260" s="2" t="s">
         <v>1205</v>
       </c>
@@ -12025,7 +12115,7 @@
         <v>1185</v>
       </c>
     </row>
-    <row r="261" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="261" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B261" s="2" t="s">
         <v>1206</v>
       </c>
@@ -12045,7 +12135,7 @@
         <v>1185</v>
       </c>
     </row>
-    <row r="262" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="262" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B262" s="2" t="s">
         <v>1207</v>
       </c>
@@ -12065,7 +12155,7 @@
         <v>1212</v>
       </c>
     </row>
-    <row r="263" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="263" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B263" s="2" t="s">
         <v>1213</v>
       </c>
@@ -12085,7 +12175,7 @@
         <v>1218</v>
       </c>
     </row>
-    <row r="264" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="264" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B264" s="2" t="s">
         <v>1219</v>
       </c>
@@ -12105,7 +12195,7 @@
         <v>1224</v>
       </c>
     </row>
-    <row r="265" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="265" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B265" s="2" t="s">
         <v>1225</v>
       </c>
@@ -12125,7 +12215,7 @@
         <v>1230</v>
       </c>
     </row>
-    <row r="266" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="266" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B266" s="2" t="s">
         <v>1231</v>
       </c>
@@ -12145,7 +12235,7 @@
         <v>1235</v>
       </c>
     </row>
-    <row r="267" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="267" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B267" s="2" t="s">
         <v>1236</v>
       </c>
@@ -12165,7 +12255,7 @@
         <v>1240</v>
       </c>
     </row>
-    <row r="268" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="268" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B268" s="2" t="s">
         <v>1241</v>
       </c>
@@ -12185,7 +12275,7 @@
         <v>1246</v>
       </c>
     </row>
-    <row r="269" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="269" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B269" s="2" t="s">
         <v>1247</v>
       </c>
@@ -12205,7 +12295,7 @@
         <v>1246</v>
       </c>
     </row>
-    <row r="270" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="270" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B270" s="2" t="s">
         <v>1248</v>
       </c>
@@ -12225,7 +12315,7 @@
         <v>1246</v>
       </c>
     </row>
-    <row r="271" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="271" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B271" s="2" t="s">
         <v>1249</v>
       </c>
@@ -12245,7 +12335,7 @@
         <v>1246</v>
       </c>
     </row>
-    <row r="272" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="272" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B272" s="2" t="s">
         <v>1250</v>
       </c>
@@ -12265,7 +12355,7 @@
         <v>1255</v>
       </c>
     </row>
-    <row r="273" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="273" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B273" s="2" t="s">
         <v>1256</v>
       </c>
@@ -12285,7 +12375,7 @@
         <v>1235</v>
       </c>
     </row>
-    <row r="274" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="274" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B274" s="2" t="s">
         <v>1257</v>
       </c>
@@ -12305,7 +12395,7 @@
         <v>1240</v>
       </c>
     </row>
-    <row r="275" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="275" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B275" s="2" t="s">
         <v>1258</v>
       </c>
@@ -12325,7 +12415,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="276" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="276" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B276" s="2" t="s">
         <v>1259</v>
       </c>
@@ -12345,7 +12435,7 @@
         <v>1264</v>
       </c>
     </row>
-    <row r="277" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="277" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B277" s="2" t="s">
         <v>1265</v>
       </c>
@@ -12365,7 +12455,7 @@
         <v>1270</v>
       </c>
     </row>
-    <row r="278" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="278" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B278" s="2" t="s">
         <v>1271</v>
       </c>
@@ -12385,7 +12475,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="279" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="279" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B279" s="2" t="s">
         <v>1272</v>
       </c>
@@ -12405,7 +12495,7 @@
         <v>1277</v>
       </c>
     </row>
-    <row r="280" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="280" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B280" s="2" t="s">
         <v>1278</v>
       </c>
@@ -12425,7 +12515,7 @@
         <v>1283</v>
       </c>
     </row>
-    <row r="281" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="281" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B281" s="2" t="s">
         <v>1284</v>
       </c>
@@ -12445,7 +12535,7 @@
         <v>1287</v>
       </c>
     </row>
-    <row r="282" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="282" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B282" s="2" t="s">
         <v>1288</v>
       </c>
@@ -12465,7 +12555,7 @@
         <v>1292</v>
       </c>
     </row>
-    <row r="283" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="283" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B283" s="2" t="s">
         <v>1293</v>
       </c>
@@ -12485,7 +12575,7 @@
         <v>1298</v>
       </c>
     </row>
-    <row r="284" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="284" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B284" s="2" t="s">
         <v>1299</v>
       </c>
@@ -12505,7 +12595,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="285" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="285" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B285" s="2" t="s">
         <v>1305</v>
       </c>
@@ -12525,7 +12615,7 @@
         <v>1310</v>
       </c>
     </row>
-    <row r="286" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="286" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B286" s="2" t="s">
         <v>1311</v>
       </c>
@@ -12545,7 +12635,7 @@
         <v>1316</v>
       </c>
     </row>
-    <row r="287" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="287" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B287" s="2" t="s">
         <v>1317</v>
       </c>
@@ -12565,7 +12655,7 @@
         <v>1316</v>
       </c>
     </row>
-    <row r="288" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="288" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B288" s="2" t="s">
         <v>1318</v>
       </c>
@@ -12585,7 +12675,7 @@
         <v>1323</v>
       </c>
     </row>
-    <row r="289" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="289" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B289" s="2" t="s">
         <v>1324</v>
       </c>
@@ -12605,7 +12695,7 @@
         <v>1323</v>
       </c>
     </row>
-    <row r="290" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="290" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B290" s="2" t="s">
         <v>1325</v>
       </c>
@@ -12625,7 +12715,7 @@
         <v>1329</v>
       </c>
     </row>
-    <row r="291" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="291" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B291" s="2" t="s">
         <v>1330</v>
       </c>
@@ -12645,7 +12735,7 @@
         <v>1329</v>
       </c>
     </row>
-    <row r="292" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="292" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B292" s="2"/>
       <c r="C292" s="2"/>
       <c r="D292" s="2"/>
@@ -12653,7 +12743,7 @@
       <c r="F292" s="2"/>
       <c r="G292" s="2"/>
     </row>
-    <row r="293" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="293" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B293" s="2"/>
       <c r="C293" s="2"/>
       <c r="D293" s="2"/>
@@ -12661,7 +12751,7 @@
       <c r="F293" s="2"/>
       <c r="G293" s="2"/>
     </row>
-    <row r="294" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="294" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B294" s="3" t="s">
         <v>1331</v>
       </c>
@@ -12671,7 +12761,7 @@
       <c r="F294" s="2"/>
       <c r="G294" s="2"/>
     </row>
-    <row r="295" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="295" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B295" s="2"/>
       <c r="C295" s="2"/>
       <c r="D295" s="2"/>
@@ -12679,7 +12769,7 @@
       <c r="F295" s="2"/>
       <c r="G295" s="2"/>
     </row>
-    <row r="296" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="296" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B296" s="2" t="s">
         <v>3</v>
       </c>
@@ -12699,7 +12789,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="297" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="297" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B297" s="2" t="s">
         <v>1332</v>
       </c>
@@ -12719,7 +12809,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="298" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="298" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B298" s="2" t="s">
         <v>1334</v>
       </c>
@@ -12739,7 +12829,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="299" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="299" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B299" s="2" t="s">
         <v>1337</v>
       </c>
@@ -12759,7 +12849,7 @@
         <v>1342</v>
       </c>
     </row>
-    <row r="300" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="300" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B300" s="2" t="s">
         <v>1343</v>
       </c>
@@ -12779,7 +12869,7 @@
         <v>1346</v>
       </c>
     </row>
-    <row r="301" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="301" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B301" s="2" t="s">
         <v>1347</v>
       </c>
@@ -12799,7 +12889,7 @@
         <v>1349</v>
       </c>
     </row>
-    <row r="302" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="302" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B302" s="2" t="s">
         <v>1350</v>
       </c>
@@ -12819,7 +12909,7 @@
         <v>1355</v>
       </c>
     </row>
-    <row r="303" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="303" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B303" s="2" t="s">
         <v>1356</v>
       </c>
@@ -12839,7 +12929,7 @@
         <v>1361</v>
       </c>
     </row>
-    <row r="304" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="304" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B304" s="2" t="s">
         <v>1362</v>
       </c>
@@ -12859,7 +12949,7 @@
         <v>1367</v>
       </c>
     </row>
-    <row r="305" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="305" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B305" s="2" t="s">
         <v>1368</v>
       </c>
@@ -12879,7 +12969,7 @@
         <v>2006</v>
       </c>
     </row>
-    <row r="306" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="306" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B306" s="2" t="s">
         <v>1369</v>
       </c>
@@ -12899,7 +12989,7 @@
         <v>1118</v>
       </c>
     </row>
-    <row r="307" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="307" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B307" s="2" t="s">
         <v>1372</v>
       </c>
@@ -12919,7 +13009,7 @@
         <v>1376</v>
       </c>
     </row>
-    <row r="308" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="308" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B308" s="2" t="s">
         <v>1377</v>
       </c>
@@ -12939,7 +13029,7 @@
         <v>1382</v>
       </c>
     </row>
-    <row r="309" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="309" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B309" s="2" t="s">
         <v>1383</v>
       </c>
@@ -12959,7 +13049,7 @@
         <v>1388</v>
       </c>
     </row>
-    <row r="310" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="310" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B310" s="2" t="s">
         <v>1389</v>
       </c>
@@ -12979,7 +13069,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="311" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="311" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B311" s="2" t="s">
         <v>1390</v>
       </c>
@@ -12999,7 +13089,7 @@
         <v>1019</v>
       </c>
     </row>
-    <row r="312" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="312" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B312" s="2" t="s">
         <v>1391</v>
       </c>
@@ -13019,7 +13109,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="313" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="313" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B313" s="2" t="s">
         <v>1394</v>
       </c>
@@ -13039,7 +13129,7 @@
         <v>1398</v>
       </c>
     </row>
-    <row r="314" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="314" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B314" s="2" t="s">
         <v>1399</v>
       </c>
@@ -13059,7 +13149,7 @@
         <v>1404</v>
       </c>
     </row>
-    <row r="315" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="315" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B315" s="2" t="s">
         <v>1405</v>
       </c>
@@ -13079,7 +13169,7 @@
         <v>1410</v>
       </c>
     </row>
-    <row r="316" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="316" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B316" s="2" t="s">
         <v>1411</v>
       </c>
@@ -13099,7 +13189,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="317" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="317" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B317" s="2" t="s">
         <v>1412</v>
       </c>
@@ -13119,7 +13209,7 @@
         <v>1417</v>
       </c>
     </row>
-    <row r="318" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="318" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B318" s="2" t="s">
         <v>1418</v>
       </c>
@@ -13139,7 +13229,7 @@
         <v>1423</v>
       </c>
     </row>
-    <row r="319" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="319" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B319" s="2" t="s">
         <v>1424</v>
       </c>
@@ -13159,7 +13249,7 @@
         <v>1429</v>
       </c>
     </row>
-    <row r="320" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="320" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B320" s="2" t="s">
         <v>1430</v>
       </c>
@@ -13179,7 +13269,7 @@
         <v>1435</v>
       </c>
     </row>
-    <row r="321" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="321" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B321" s="2" t="s">
         <v>1436</v>
       </c>
@@ -13199,7 +13289,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="322" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="322" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B322" s="2" t="s">
         <v>1442</v>
       </c>
@@ -13219,7 +13309,7 @@
         <v>1447</v>
       </c>
     </row>
-    <row r="323" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="323" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B323" s="2" t="s">
         <v>1448</v>
       </c>
@@ -13239,7 +13329,7 @@
         <v>1451</v>
       </c>
     </row>
-    <row r="324" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="324" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B324" s="2" t="s">
         <v>1452</v>
       </c>
@@ -13259,7 +13349,7 @@
         <v>1457</v>
       </c>
     </row>
-    <row r="325" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="325" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B325" s="2" t="s">
         <v>1458</v>
       </c>
@@ -13279,7 +13369,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="326" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="326" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B326" s="2" t="s">
         <v>1459</v>
       </c>
@@ -13299,7 +13389,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="327" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="327" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B327" s="2" t="s">
         <v>1460</v>
       </c>
@@ -13319,7 +13409,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="328" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="328" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B328" s="2" t="s">
         <v>1461</v>
       </c>
@@ -13339,7 +13429,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="329" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="329" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B329" s="2" t="s">
         <v>1463</v>
       </c>
@@ -13359,7 +13449,7 @@
         <v>1468</v>
       </c>
     </row>
-    <row r="330" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="330" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B330" s="2" t="s">
         <v>1469</v>
       </c>
@@ -13379,7 +13469,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="331" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="331" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B331" s="2" t="s">
         <v>1470</v>
       </c>
@@ -13399,7 +13489,7 @@
         <v>1475</v>
       </c>
     </row>
-    <row r="332" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="332" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B332" s="2" t="s">
         <v>1476</v>
       </c>
@@ -13419,7 +13509,7 @@
         <v>1480</v>
       </c>
     </row>
-    <row r="333" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="333" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B333" s="2" t="s">
         <v>1481</v>
       </c>
@@ -13439,7 +13529,7 @@
         <v>1482</v>
       </c>
     </row>
-    <row r="334" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="334" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B334" s="2" t="s">
         <v>1483</v>
       </c>
@@ -13474,13 +13564,13 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="B2:G114"/>
-  <sheetFormatPr defaultColWidth="12" defaultRowHeight="12" x14ac:dyDescent="0.2"/>
+  <dimension ref="B2:G121"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
   <cols>
-    <col min="1" max="200" width="35.6640625" customWidth="1"/>
+    <col min="1" max="200" width="35.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
@@ -13490,7 +13580,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -13498,7 +13588,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B4" s="3" t="s">
         <v>1489</v>
       </c>
@@ -13508,7 +13598,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -13516,7 +13606,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
@@ -13536,7 +13626,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B7" s="2" t="s">
         <v>1827</v>
       </c>
@@ -13556,7 +13646,7 @@
         <v>1107</v>
       </c>
     </row>
-    <row r="8" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B8" s="2" t="s">
         <v>1579</v>
       </c>
@@ -13576,7 +13666,7 @@
         <v>1584</v>
       </c>
     </row>
-    <row r="9" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B9" s="2" t="s">
         <v>1781</v>
       </c>
@@ -13596,7 +13686,7 @@
         <v>1786</v>
       </c>
     </row>
-    <row r="10" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B10" s="2" t="s">
         <v>1598</v>
       </c>
@@ -13616,7 +13706,7 @@
         <v>1603</v>
       </c>
     </row>
-    <row r="11" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B11" s="2" t="s">
         <v>1495</v>
       </c>
@@ -13636,7 +13726,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="12" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B12" s="2" t="s">
         <v>1536</v>
       </c>
@@ -13656,7 +13746,7 @@
         <v>1541</v>
       </c>
     </row>
-    <row r="13" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B13" s="2" t="s">
         <v>1639</v>
       </c>
@@ -13676,7 +13766,7 @@
         <v>1643</v>
       </c>
     </row>
-    <row r="14" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B14" s="2" t="s">
         <v>1654</v>
       </c>
@@ -13696,7 +13786,7 @@
         <v>1659</v>
       </c>
     </row>
-    <row r="15" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B15" s="2" t="s">
         <v>1775</v>
       </c>
@@ -13716,7 +13806,7 @@
         <v>1780</v>
       </c>
     </row>
-    <row r="16" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B16" s="2" t="s">
         <v>1665</v>
       </c>
@@ -13736,7 +13826,7 @@
         <v>1666</v>
       </c>
     </row>
-    <row r="17" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B17" s="2" t="s">
         <v>1627</v>
       </c>
@@ -13756,7 +13846,7 @@
         <v>1632</v>
       </c>
     </row>
-    <row r="18" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B18" s="2" t="s">
         <v>1787</v>
       </c>
@@ -13776,7 +13866,7 @@
         <v>1791</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B19" s="2" t="s">
         <v>1792</v>
       </c>
@@ -13796,7 +13886,7 @@
         <v>1797</v>
       </c>
     </row>
-    <row r="20" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="20" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B20" s="2" t="s">
         <v>1519</v>
       </c>
@@ -13816,7 +13906,7 @@
         <v>1524</v>
       </c>
     </row>
-    <row r="21" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B21" s="2" t="s">
         <v>1501</v>
       </c>
@@ -13836,7 +13926,7 @@
         <v>1506</v>
       </c>
     </row>
-    <row r="22" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B22" s="2" t="s">
         <v>1741</v>
       </c>
@@ -13856,7 +13946,7 @@
         <v>1742</v>
       </c>
     </row>
-    <row r="23" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B23" s="2" t="s">
         <v>1490</v>
       </c>
@@ -13876,7 +13966,7 @@
         <v>1491</v>
       </c>
     </row>
-    <row r="24" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="24" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B24" s="2" t="s">
         <v>1682</v>
       </c>
@@ -13896,7 +13986,7 @@
         <v>1687</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B25" s="2" t="s">
         <v>274</v>
       </c>
@@ -13916,7 +14006,7 @@
         <v>1561</v>
       </c>
     </row>
-    <row r="26" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B26" s="2" t="s">
         <v>1591</v>
       </c>
@@ -13936,7 +14026,7 @@
         <v>1561</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B27" s="2" t="s">
         <v>1568</v>
       </c>
@@ -13956,7 +14046,7 @@
         <v>1573</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="28" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B28" s="2" t="s">
         <v>1548</v>
       </c>
@@ -13976,7 +14066,7 @@
         <v>1553</v>
       </c>
     </row>
-    <row r="29" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="29" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B29" s="2" t="s">
         <v>399</v>
       </c>
@@ -13996,7 +14086,7 @@
         <v>1578</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B30" s="2" t="s">
         <v>1729</v>
       </c>
@@ -14016,7 +14106,7 @@
         <v>1734</v>
       </c>
     </row>
-    <row r="31" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B31" s="2" t="s">
         <v>1585</v>
       </c>
@@ -14036,7 +14126,7 @@
         <v>1590</v>
       </c>
     </row>
-    <row r="32" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="32" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B32" s="2" t="s">
         <v>1735</v>
       </c>
@@ -14056,7 +14146,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="33" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B33" s="2" t="s">
         <v>1763</v>
       </c>
@@ -14076,7 +14166,7 @@
         <v>1768</v>
       </c>
     </row>
-    <row r="34" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B34" s="2" t="s">
         <v>1821</v>
       </c>
@@ -14096,7 +14186,7 @@
         <v>1826</v>
       </c>
     </row>
-    <row r="35" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B35" s="2" t="s">
         <v>1798</v>
       </c>
@@ -14116,7 +14206,7 @@
         <v>1803</v>
       </c>
     </row>
-    <row r="36" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="36" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B36" s="2" t="s">
         <v>1804</v>
       </c>
@@ -14136,7 +14226,7 @@
         <v>1808</v>
       </c>
     </row>
-    <row r="37" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B37" s="2" t="s">
         <v>1815</v>
       </c>
@@ -14156,7 +14246,7 @@
         <v>1820</v>
       </c>
     </row>
-    <row r="38" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="38" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B38" s="2" t="s">
         <v>1700</v>
       </c>
@@ -14176,7 +14266,7 @@
         <v>1705</v>
       </c>
     </row>
-    <row r="39" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B39" s="2" t="s">
         <v>1828</v>
       </c>
@@ -14196,7 +14286,7 @@
         <v>1829</v>
       </c>
     </row>
-    <row r="40" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="40" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B40" s="4" t="s">
         <v>2024</v>
       </c>
@@ -14216,7 +14306,7 @@
         <v>2029</v>
       </c>
     </row>
-    <row r="41" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B41" s="2" t="s">
         <v>1836</v>
       </c>
@@ -14236,7 +14326,7 @@
         <v>1841</v>
       </c>
     </row>
-    <row r="42" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="42" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B42" s="2" t="s">
         <v>1513</v>
       </c>
@@ -14256,7 +14346,7 @@
         <v>1518</v>
       </c>
     </row>
-    <row r="43" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="43" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B43" s="2" t="s">
         <v>1830</v>
       </c>
@@ -14276,7 +14366,7 @@
         <v>1835</v>
       </c>
     </row>
-    <row r="44" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="44" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B44" s="2" t="s">
         <v>1621</v>
       </c>
@@ -14296,7 +14386,7 @@
         <v>1626</v>
       </c>
     </row>
-    <row r="45" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B45" s="2" t="s">
         <v>1649</v>
       </c>
@@ -14316,7 +14406,7 @@
         <v>1650</v>
       </c>
     </row>
-    <row r="46" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="46" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B46" s="2" t="s">
         <v>1809</v>
       </c>
@@ -14336,7 +14426,7 @@
         <v>1814</v>
       </c>
     </row>
-    <row r="47" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B47" s="2" t="s">
         <v>1644</v>
       </c>
@@ -14356,7 +14446,7 @@
         <v>1645</v>
       </c>
     </row>
-    <row r="48" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="48" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B48" s="2" t="s">
         <v>1736</v>
       </c>
@@ -14376,7 +14466,7 @@
         <v>1737</v>
       </c>
     </row>
-    <row r="49" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B49" s="2" t="s">
         <v>1745</v>
       </c>
@@ -14396,7 +14486,7 @@
         <v>1750</v>
       </c>
     </row>
-    <row r="50" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="50" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B50" s="2" t="s">
         <v>1615</v>
       </c>
@@ -14416,7 +14506,7 @@
         <v>1620</v>
       </c>
     </row>
-    <row r="51" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B51" s="2" t="s">
         <v>558</v>
       </c>
@@ -14436,7 +14526,7 @@
         <v>1614</v>
       </c>
     </row>
-    <row r="52" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="52" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B52" s="2" t="s">
         <v>1507</v>
       </c>
@@ -14456,7 +14546,7 @@
         <v>1512</v>
       </c>
     </row>
-    <row r="53" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B53" s="2" t="s">
         <v>1525</v>
       </c>
@@ -14476,7 +14566,7 @@
         <v>1530</v>
       </c>
     </row>
-    <row r="54" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="54" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B54" s="2" t="s">
         <v>1670</v>
       </c>
@@ -14496,7 +14586,7 @@
         <v>1675</v>
       </c>
     </row>
-    <row r="55" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B55" s="2" t="s">
         <v>1562</v>
       </c>
@@ -14516,7 +14606,7 @@
         <v>1567</v>
       </c>
     </row>
-    <row r="56" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="56" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B56" s="2" t="s">
         <v>1676</v>
       </c>
@@ -14536,7 +14626,7 @@
         <v>1681</v>
       </c>
     </row>
-    <row r="57" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B57" s="2" t="s">
         <v>1688</v>
       </c>
@@ -14556,7 +14646,7 @@
         <v>1693</v>
       </c>
     </row>
-    <row r="58" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="58" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B58" s="2" t="s">
         <v>1694</v>
       </c>
@@ -14576,7 +14666,7 @@
         <v>1699</v>
       </c>
     </row>
-    <row r="59" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B59" s="2" t="s">
         <v>1706</v>
       </c>
@@ -14596,7 +14686,7 @@
         <v>1711</v>
       </c>
     </row>
-    <row r="60" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="60" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B60" s="2" t="s">
         <v>1712</v>
       </c>
@@ -14616,7 +14706,7 @@
         <v>1717</v>
       </c>
     </row>
-    <row r="61" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B61" s="2" t="s">
         <v>1718</v>
       </c>
@@ -14636,7 +14726,7 @@
         <v>1723</v>
       </c>
     </row>
-    <row r="62" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="62" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B62" s="2" t="s">
         <v>1542</v>
       </c>
@@ -14656,7 +14746,7 @@
         <v>1547</v>
       </c>
     </row>
-    <row r="63" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B63" s="2" t="s">
         <v>1592</v>
       </c>
@@ -14676,7 +14766,7 @@
         <v>1597</v>
       </c>
     </row>
-    <row r="64" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="64" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B64" s="2" t="s">
         <v>1531</v>
       </c>
@@ -14696,7 +14786,7 @@
         <v>1532</v>
       </c>
     </row>
-    <row r="65" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B65" s="2" t="s">
         <v>1604</v>
       </c>
@@ -14716,7 +14806,7 @@
         <v>1609</v>
       </c>
     </row>
-    <row r="66" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="66" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B66" s="2" t="s">
         <v>1724</v>
       </c>
@@ -14736,7 +14826,7 @@
         <v>1725</v>
       </c>
     </row>
-    <row r="67" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B67" s="2" t="s">
         <v>1660</v>
       </c>
@@ -14756,7 +14846,7 @@
         <v>1661</v>
       </c>
     </row>
-    <row r="68" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="68" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B68" s="2" t="s">
         <v>1751</v>
       </c>
@@ -14776,7 +14866,7 @@
         <v>1756</v>
       </c>
     </row>
-    <row r="69" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B69" s="2" t="s">
         <v>1757</v>
       </c>
@@ -14796,7 +14886,7 @@
         <v>1762</v>
       </c>
     </row>
-    <row r="70" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="70" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B70" s="2" t="s">
         <v>1633</v>
       </c>
@@ -14816,7 +14906,7 @@
         <v>1638</v>
       </c>
     </row>
-    <row r="71" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
       <c r="B71" s="2" t="s">
         <v>1554</v>
       </c>
@@ -14836,7 +14926,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="72" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="72" spans="2:7" ht="39" x14ac:dyDescent="0.15">
       <c r="B72" s="2" t="s">
         <v>1769</v>
       </c>
@@ -14856,680 +14946,821 @@
         <v>1774</v>
       </c>
     </row>
-    <row r="73" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B73" s="2"/>
-      <c r="C73" s="2"/>
-      <c r="D73" s="2"/>
-      <c r="E73" s="2"/>
-      <c r="F73" s="2"/>
-      <c r="G73" s="2"/>
-    </row>
-    <row r="74" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B74" s="3" t="s">
+    <row r="73" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B73" s="4" t="s">
+        <v>2045</v>
+      </c>
+      <c r="C73" s="4" t="s">
+        <v>2046</v>
+      </c>
+      <c r="D73" s="4" t="s">
+        <v>2047</v>
+      </c>
+      <c r="E73" s="2" t="s">
+        <v>2049</v>
+      </c>
+      <c r="F73" s="2" t="s">
+        <v>2050</v>
+      </c>
+      <c r="G73" s="2" t="s">
+        <v>2048</v>
+      </c>
+    </row>
+    <row r="74" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B74" s="4" t="s">
+        <v>2051</v>
+      </c>
+      <c r="C74" s="4" t="s">
+        <v>1344</v>
+      </c>
+      <c r="D74" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="E74" t="s">
+        <v>12</v>
+      </c>
+      <c r="F74" t="s">
+        <v>13</v>
+      </c>
+      <c r="G74" t="s">
+        <v>2062</v>
+      </c>
+    </row>
+    <row r="75" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B75" s="4" t="s">
+        <v>2052</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>2053</v>
+      </c>
+      <c r="D75" s="4" t="s">
+        <v>2054</v>
+      </c>
+      <c r="E75" s="2" t="s">
+        <v>2064</v>
+      </c>
+      <c r="F75" s="2" t="s">
+        <v>2065</v>
+      </c>
+      <c r="G75" s="2" t="s">
+        <v>2063</v>
+      </c>
+    </row>
+    <row r="76" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B76" s="4" t="s">
+        <v>2055</v>
+      </c>
+      <c r="C76" s="4" t="s">
+        <v>2056</v>
+      </c>
+      <c r="D76" s="4" t="s">
+        <v>2057</v>
+      </c>
+      <c r="E76" s="2" t="s">
+        <v>2060</v>
+      </c>
+      <c r="F76" s="2" t="s">
+        <v>2059</v>
+      </c>
+      <c r="G76" s="2" t="s">
+        <v>2061</v>
+      </c>
+    </row>
+    <row r="77" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B77" s="4" t="s">
+        <v>2058</v>
+      </c>
+      <c r="C77" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D77" s="4" t="s">
+        <v>1005</v>
+      </c>
+      <c r="E77" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F77" t="s">
+        <v>35</v>
+      </c>
+      <c r="G77" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="78" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B78" s="8" t="s">
+        <v>2066</v>
+      </c>
+      <c r="C78" s="8" t="s">
+        <v>1816</v>
+      </c>
+      <c r="D78" s="8" t="s">
+        <v>1817</v>
+      </c>
+      <c r="E78" s="8" t="s">
+        <v>1819</v>
+      </c>
+      <c r="F78" t="s">
+        <v>1818</v>
+      </c>
+      <c r="G78" s="8" t="s">
+        <v>1820</v>
+      </c>
+    </row>
+    <row r="79" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B79" s="8" t="s">
+        <v>2067</v>
+      </c>
+      <c r="C79" s="8" t="s">
+        <v>2068</v>
+      </c>
+      <c r="D79" s="8" t="s">
+        <v>2069</v>
+      </c>
+      <c r="E79" s="8" t="s">
+        <v>2070</v>
+      </c>
+      <c r="F79" t="s">
+        <v>2070</v>
+      </c>
+      <c r="G79" s="8" t="s">
+        <v>2071</v>
+      </c>
+    </row>
+    <row r="80" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B80" s="2"/>
+      <c r="C80" s="2"/>
+      <c r="D80" s="2"/>
+      <c r="E80" s="2"/>
+      <c r="F80" s="2"/>
+      <c r="G80" s="2"/>
+    </row>
+    <row r="81" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B81" s="3" t="s">
         <v>1842</v>
       </c>
-      <c r="C74" s="2"/>
-      <c r="D74" s="2"/>
-      <c r="E74" s="2"/>
-      <c r="F74" s="2"/>
-      <c r="G74" s="2"/>
-    </row>
-    <row r="75" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B75" s="2"/>
-      <c r="C75" s="2"/>
-      <c r="D75" s="2"/>
-      <c r="E75" s="2"/>
-      <c r="F75" s="2"/>
-      <c r="G75" s="2"/>
-    </row>
-    <row r="76" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B76" s="2" t="s">
+      <c r="C81" s="2"/>
+      <c r="D81" s="2"/>
+      <c r="E81" s="2"/>
+      <c r="F81" s="2"/>
+      <c r="G81" s="2"/>
+    </row>
+    <row r="82" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B82" s="2"/>
+      <c r="C82" s="2"/>
+      <c r="D82" s="2"/>
+      <c r="E82" s="2"/>
+      <c r="F82" s="2"/>
+      <c r="G82" s="2"/>
+    </row>
+    <row r="83" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B83" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C76" s="2" t="s">
+      <c r="C83" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D76" s="2" t="s">
+      <c r="D83" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E76" s="2" t="s">
+      <c r="E83" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F76" s="2" t="s">
+      <c r="F83" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G76" s="2" t="s">
+      <c r="G83" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="77" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B77" s="2" t="s">
+    <row r="84" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B84" s="2" t="s">
         <v>1843</v>
       </c>
-      <c r="C77" s="2" t="s">
+      <c r="C84" s="2" t="s">
         <v>1844</v>
       </c>
-      <c r="D77" s="2" t="s">
+      <c r="D84" s="2" t="s">
         <v>1845</v>
       </c>
-      <c r="E77" s="2" t="s">
+      <c r="E84" s="2" t="s">
         <v>1846</v>
       </c>
-      <c r="F77" s="2" t="s">
+      <c r="F84" s="2" t="s">
         <v>1847</v>
       </c>
-      <c r="G77" s="2" t="s">
+      <c r="G84" s="2" t="s">
         <v>1848</v>
       </c>
     </row>
-    <row r="78" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B78" s="2" t="s">
+    <row r="85" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B85" s="2" t="s">
         <v>1849</v>
       </c>
-      <c r="C78" s="2" t="s">
+      <c r="C85" s="2" t="s">
         <v>1850</v>
       </c>
-      <c r="D78" s="2" t="s">
+      <c r="D85" s="2" t="s">
         <v>1850</v>
       </c>
-      <c r="E78" s="2" t="s">
+      <c r="E85" s="2" t="s">
         <v>1851</v>
       </c>
-      <c r="F78" s="2" t="s">
+      <c r="F85" s="2" t="s">
         <v>1852</v>
       </c>
-      <c r="G78" s="2" t="s">
+      <c r="G85" s="2" t="s">
         <v>1853</v>
       </c>
     </row>
-    <row r="79" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B79" s="2" t="s">
+    <row r="86" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B86" s="2" t="s">
         <v>1854</v>
       </c>
-      <c r="C79" s="2" t="s">
+      <c r="C86" s="2" t="s">
         <v>1855</v>
       </c>
-      <c r="D79" s="2" t="s">
+      <c r="D86" s="2" t="s">
         <v>1856</v>
       </c>
-      <c r="E79" s="2" t="s">
+      <c r="E86" s="2" t="s">
         <v>1857</v>
       </c>
-      <c r="F79" s="2" t="s">
+      <c r="F86" s="2" t="s">
         <v>1858</v>
       </c>
-      <c r="G79" s="2" t="s">
+      <c r="G86" s="2" t="s">
         <v>1859</v>
       </c>
     </row>
-    <row r="80" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B80" s="2" t="s">
+    <row r="87" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B87" s="2" t="s">
         <v>1860</v>
       </c>
-      <c r="C80" s="2" t="s">
+      <c r="C87" s="2" t="s">
         <v>1861</v>
       </c>
-      <c r="D80" s="2" t="s">
+      <c r="D87" s="2" t="s">
         <v>1862</v>
       </c>
-      <c r="E80" s="2" t="s">
+      <c r="E87" s="2" t="s">
         <v>1863</v>
       </c>
-      <c r="F80" s="2" t="s">
+      <c r="F87" s="2" t="s">
         <v>1864</v>
       </c>
-      <c r="G80" s="2" t="s">
+      <c r="G87" s="2" t="s">
         <v>1865</v>
       </c>
     </row>
-    <row r="81" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B81" s="2" t="s">
+    <row r="88" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B88" s="2" t="s">
         <v>1866</v>
       </c>
-      <c r="C81" s="2" t="s">
+      <c r="C88" s="2" t="s">
         <v>1867</v>
       </c>
-      <c r="D81" s="2" t="s">
+      <c r="D88" s="2" t="s">
         <v>1868</v>
       </c>
-      <c r="E81" s="2" t="s">
+      <c r="E88" s="2" t="s">
         <v>1869</v>
       </c>
-      <c r="F81" s="2" t="s">
+      <c r="F88" s="2" t="s">
         <v>1870</v>
       </c>
-      <c r="G81" s="2" t="s">
+      <c r="G88" s="2" t="s">
         <v>1871</v>
       </c>
     </row>
-    <row r="82" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B82" s="2" t="s">
+    <row r="89" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B89" s="2" t="s">
         <v>1872</v>
       </c>
-      <c r="C82" s="2" t="s">
+      <c r="C89" s="2" t="s">
         <v>1873</v>
       </c>
-      <c r="D82" s="2" t="s">
+      <c r="D89" s="2" t="s">
         <v>1874</v>
       </c>
-      <c r="E82" s="2" t="s">
+      <c r="E89" s="2" t="s">
         <v>1875</v>
       </c>
-      <c r="F82" s="2" t="s">
+      <c r="F89" s="2" t="s">
         <v>1876</v>
       </c>
-      <c r="G82" s="2" t="s">
+      <c r="G89" s="2" t="s">
         <v>1877</v>
       </c>
     </row>
-    <row r="83" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B83" s="2" t="s">
+    <row r="90" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B90" s="2" t="s">
         <v>1878</v>
       </c>
-      <c r="C83" s="2" t="s">
+      <c r="C90" s="2" t="s">
         <v>1879</v>
       </c>
-      <c r="D83" s="2" t="s">
+      <c r="D90" s="2" t="s">
         <v>1880</v>
       </c>
-      <c r="E83" s="2" t="s">
+      <c r="E90" s="2" t="s">
         <v>1881</v>
       </c>
-      <c r="F83" s="2" t="s">
+      <c r="F90" s="2" t="s">
         <v>1882</v>
       </c>
-      <c r="G83" s="2" t="s">
+      <c r="G90" s="2" t="s">
         <v>1883</v>
       </c>
     </row>
-    <row r="84" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B84" s="2" t="s">
+    <row r="91" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B91" s="2" t="s">
         <v>1884</v>
       </c>
-      <c r="C84" s="2" t="s">
+      <c r="C91" s="2" t="s">
         <v>1885</v>
       </c>
-      <c r="D84" s="2" t="s">
+      <c r="D91" s="2" t="s">
         <v>1886</v>
       </c>
-      <c r="E84" s="2" t="s">
+      <c r="E91" s="2" t="s">
         <v>1887</v>
       </c>
-      <c r="F84" s="2" t="s">
+      <c r="F91" s="2" t="s">
         <v>1888</v>
       </c>
-      <c r="G84" s="2" t="s">
+      <c r="G91" s="2" t="s">
         <v>1889</v>
       </c>
     </row>
-    <row r="85" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B85" s="2" t="s">
+    <row r="92" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B92" s="2" t="s">
         <v>1890</v>
       </c>
-      <c r="C85" s="2" t="s">
+      <c r="C92" s="2" t="s">
         <v>1891</v>
       </c>
-      <c r="D85" s="2" t="s">
+      <c r="D92" s="2" t="s">
         <v>1892</v>
       </c>
-      <c r="E85" s="2" t="s">
+      <c r="E92" s="2" t="s">
         <v>1893</v>
       </c>
-      <c r="F85" s="2" t="s">
+      <c r="F92" s="2" t="s">
         <v>1894</v>
       </c>
-      <c r="G85" s="2" t="s">
+      <c r="G92" s="2" t="s">
         <v>1895</v>
       </c>
     </row>
-    <row r="86" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B86" s="2" t="s">
+    <row r="93" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B93" s="2" t="s">
         <v>1896</v>
       </c>
-      <c r="C86" s="2" t="s">
+      <c r="C93" s="2" t="s">
         <v>1837</v>
       </c>
-      <c r="D86" s="2" t="s">
+      <c r="D93" s="2" t="s">
         <v>1897</v>
       </c>
-      <c r="E86" s="2" t="s">
+      <c r="E93" s="2" t="s">
         <v>1898</v>
       </c>
-      <c r="F86" s="2" t="s">
+      <c r="F93" s="2" t="s">
         <v>1899</v>
       </c>
-      <c r="G86" s="2" t="s">
+      <c r="G93" s="2" t="s">
         <v>1841</v>
       </c>
     </row>
-    <row r="87" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B87" s="2" t="s">
+    <row r="94" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B94" s="2" t="s">
         <v>1900</v>
       </c>
-      <c r="C87" s="2" t="s">
+      <c r="C94" s="2" t="s">
         <v>1901</v>
       </c>
-      <c r="D87" s="2" t="s">
+      <c r="D94" s="2" t="s">
         <v>1902</v>
       </c>
-      <c r="E87" s="2" t="s">
+      <c r="E94" s="2" t="s">
         <v>1903</v>
       </c>
-      <c r="F87" s="2" t="s">
+      <c r="F94" s="2" t="s">
         <v>1904</v>
       </c>
-      <c r="G87" s="2" t="s">
+      <c r="G94" s="2" t="s">
         <v>1905</v>
       </c>
     </row>
-    <row r="88" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B88" s="2" t="s">
+    <row r="95" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B95" s="2" t="s">
         <v>1906</v>
       </c>
-      <c r="C88" s="2" t="s">
+      <c r="C95" s="2" t="s">
         <v>1907</v>
       </c>
-      <c r="D88" s="2" t="s">
+      <c r="D95" s="2" t="s">
         <v>1908</v>
       </c>
-      <c r="E88" s="2" t="s">
+      <c r="E95" s="2" t="s">
         <v>1909</v>
       </c>
-      <c r="F88" s="2" t="s">
+      <c r="F95" s="2" t="s">
         <v>1910</v>
       </c>
-      <c r="G88" s="2" t="s">
+      <c r="G95" s="2" t="s">
         <v>1911</v>
       </c>
     </row>
-    <row r="89" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B89" s="2" t="s">
+    <row r="96" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B96" s="2" t="s">
         <v>1912</v>
       </c>
-      <c r="C89" s="2" t="s">
+      <c r="C96" s="2" t="s">
         <v>1913</v>
       </c>
-      <c r="D89" s="2" t="s">
+      <c r="D96" s="2" t="s">
         <v>1914</v>
       </c>
-      <c r="E89" s="2" t="s">
+      <c r="E96" s="2" t="s">
         <v>1915</v>
       </c>
-      <c r="F89" s="2" t="s">
+      <c r="F96" s="2" t="s">
         <v>1915</v>
       </c>
-      <c r="G89" s="2" t="s">
+      <c r="G96" s="2" t="s">
         <v>1916</v>
       </c>
     </row>
-    <row r="90" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B90" s="2" t="s">
+    <row r="97" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B97" s="2" t="s">
         <v>2031</v>
       </c>
-      <c r="C90" s="2" t="s">
+      <c r="C97" s="2" t="s">
         <v>2032</v>
       </c>
-      <c r="D90" s="2" t="s">
+      <c r="D97" s="2" t="s">
         <v>2033</v>
       </c>
-      <c r="E90" s="2" t="s">
+      <c r="E97" s="2" t="s">
         <v>2034</v>
       </c>
-      <c r="F90" s="2" t="s">
+      <c r="F97" s="2" t="s">
         <v>2035</v>
       </c>
-      <c r="G90" s="2" t="s">
+      <c r="G97" s="2" t="s">
         <v>2036</v>
       </c>
     </row>
-    <row r="91" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B91" s="2"/>
-      <c r="C91" s="2"/>
-      <c r="D91" s="2"/>
-      <c r="E91" s="2"/>
-      <c r="F91" s="2"/>
-      <c r="G91" s="2"/>
-    </row>
-    <row r="92" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B92" s="3" t="s">
+    <row r="98" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B98" s="2"/>
+      <c r="C98" s="2"/>
+      <c r="D98" s="2"/>
+      <c r="E98" s="2"/>
+      <c r="F98" s="2"/>
+      <c r="G98" s="2"/>
+    </row>
+    <row r="99" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B99" s="3" t="s">
         <v>1917</v>
       </c>
-      <c r="C92" s="2"/>
-      <c r="D92" s="2"/>
-      <c r="E92" s="2"/>
-      <c r="F92" s="2"/>
-      <c r="G92" s="2"/>
-    </row>
-    <row r="93" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B93" s="2"/>
-      <c r="C93" s="2"/>
-      <c r="D93" s="2"/>
-      <c r="E93" s="2"/>
-      <c r="F93" s="2"/>
-      <c r="G93" s="2"/>
-    </row>
-    <row r="94" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B94" s="2" t="s">
+      <c r="C99" s="2"/>
+      <c r="D99" s="2"/>
+      <c r="E99" s="2"/>
+      <c r="F99" s="2"/>
+      <c r="G99" s="2"/>
+    </row>
+    <row r="100" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B100" s="2"/>
+      <c r="C100" s="2"/>
+      <c r="D100" s="2"/>
+      <c r="E100" s="2"/>
+      <c r="F100" s="2"/>
+      <c r="G100" s="2"/>
+    </row>
+    <row r="101" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B101" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C94" s="2" t="s">
+      <c r="C101" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="D94" s="2" t="s">
+      <c r="D101" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="E94" s="2" t="s">
+      <c r="E101" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="F94" s="2" t="s">
+      <c r="F101" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="G94" s="2" t="s">
+      <c r="G101" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="95" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B95" s="2" t="s">
+    <row r="102" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B102" s="2" t="s">
         <v>1918</v>
       </c>
-      <c r="C95" s="2" t="s">
+      <c r="C102" s="2" t="s">
         <v>1077</v>
       </c>
-      <c r="D95" s="2" t="s">
+      <c r="D102" s="2" t="s">
         <v>1078</v>
       </c>
-      <c r="E95" s="2" t="s">
+      <c r="E102" s="2" t="s">
         <v>1079</v>
       </c>
-      <c r="F95" s="2" t="s">
+      <c r="F102" s="2" t="s">
         <v>1079</v>
       </c>
-      <c r="G95" s="2" t="s">
+      <c r="G102" s="2" t="s">
         <v>1080</v>
       </c>
     </row>
-    <row r="96" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B96" s="2" t="s">
+    <row r="103" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B103" s="2" t="s">
         <v>1919</v>
       </c>
-      <c r="C96" s="2" t="s">
+      <c r="C103" s="2" t="s">
         <v>1920</v>
       </c>
-      <c r="D96" s="2" t="s">
+      <c r="D103" s="2" t="s">
         <v>1921</v>
       </c>
-      <c r="E96" s="2" t="s">
+      <c r="E103" s="2" t="s">
         <v>1922</v>
       </c>
-      <c r="F96" s="2" t="s">
+      <c r="F103" s="2" t="s">
         <v>1923</v>
       </c>
-      <c r="G96" s="2" t="s">
+      <c r="G103" s="2" t="s">
         <v>1924</v>
       </c>
     </row>
-    <row r="97" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B97" s="2" t="s">
+    <row r="104" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B104" s="2" t="s">
         <v>1925</v>
       </c>
-      <c r="C97" s="2" t="s">
+      <c r="C104" s="2" t="s">
         <v>1926</v>
       </c>
-      <c r="D97" s="2" t="s">
+      <c r="D104" s="2" t="s">
         <v>1927</v>
       </c>
-      <c r="E97" s="2" t="s">
+      <c r="E104" s="2" t="s">
         <v>1928</v>
       </c>
-      <c r="F97" s="2" t="s">
+      <c r="F104" s="2" t="s">
         <v>1929</v>
       </c>
-      <c r="G97" s="2" t="s">
+      <c r="G104" s="2" t="s">
         <v>1930</v>
       </c>
     </row>
-    <row r="98" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B98" s="2" t="s">
+    <row r="105" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B105" s="2" t="s">
         <v>1931</v>
       </c>
-      <c r="C98" s="2" t="s">
+      <c r="C105" s="2" t="s">
         <v>1932</v>
       </c>
-      <c r="D98" s="2" t="s">
+      <c r="D105" s="2" t="s">
         <v>1933</v>
       </c>
-      <c r="E98" s="2" t="s">
+      <c r="E105" s="2" t="s">
         <v>1934</v>
       </c>
-      <c r="F98" s="2" t="s">
+      <c r="F105" s="2" t="s">
         <v>1935</v>
       </c>
-      <c r="G98" s="2" t="s">
+      <c r="G105" s="2" t="s">
         <v>1936</v>
       </c>
     </row>
-    <row r="99" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B99" s="2" t="s">
+    <row r="106" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B106" s="2" t="s">
         <v>1937</v>
       </c>
-      <c r="C99" s="2" t="s">
+      <c r="C106" s="2" t="s">
         <v>1938</v>
       </c>
-      <c r="D99" s="2" t="s">
+      <c r="D106" s="2" t="s">
         <v>1939</v>
       </c>
-      <c r="E99" s="2" t="s">
+      <c r="E106" s="2" t="s">
         <v>1940</v>
       </c>
-      <c r="F99" s="2" t="s">
+      <c r="F106" s="2" t="s">
         <v>1941</v>
       </c>
-      <c r="G99" s="2" t="s">
+      <c r="G106" s="2" t="s">
         <v>1942</v>
       </c>
     </row>
-    <row r="100" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B100" s="2" t="s">
+    <row r="107" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B107" s="2" t="s">
         <v>1943</v>
       </c>
-      <c r="C100" s="2" t="s">
+      <c r="C107" s="2" t="s">
         <v>1944</v>
       </c>
-      <c r="D100" s="2" t="s">
+      <c r="D107" s="2" t="s">
         <v>1945</v>
       </c>
-      <c r="E100" s="2" t="s">
+      <c r="E107" s="2" t="s">
         <v>1946</v>
       </c>
-      <c r="F100" s="2" t="s">
+      <c r="F107" s="2" t="s">
         <v>1947</v>
       </c>
-      <c r="G100" s="2" t="s">
+      <c r="G107" s="2" t="s">
         <v>1948</v>
       </c>
     </row>
-    <row r="101" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B101" s="2" t="s">
+    <row r="108" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B108" s="2" t="s">
         <v>1949</v>
       </c>
-      <c r="C101" s="2" t="s">
+      <c r="C108" s="2" t="s">
         <v>1810</v>
       </c>
-      <c r="D101" s="2" t="s">
+      <c r="D108" s="2" t="s">
         <v>1950</v>
       </c>
-      <c r="E101" s="2" t="s">
+      <c r="E108" s="2" t="s">
         <v>1951</v>
       </c>
-      <c r="F101" s="2" t="s">
+      <c r="F108" s="2" t="s">
         <v>1952</v>
       </c>
-      <c r="G101" s="2" t="s">
+      <c r="G108" s="2" t="s">
         <v>1953</v>
       </c>
     </row>
-    <row r="102" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B102" s="2" t="s">
+    <row r="109" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B109" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="C102" s="2" t="s">
+      <c r="C109" s="2" t="s">
         <v>1788</v>
       </c>
-      <c r="D102" s="2" t="s">
+      <c r="D109" s="2" t="s">
         <v>1954</v>
       </c>
-      <c r="E102" s="2" t="s">
+      <c r="E109" s="2" t="s">
         <v>1955</v>
       </c>
-      <c r="F102" s="2" t="s">
+      <c r="F109" s="2" t="s">
         <v>1956</v>
       </c>
-      <c r="G102" s="2" t="s">
+      <c r="G109" s="2" t="s">
         <v>1957</v>
       </c>
     </row>
-    <row r="103" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B103" s="2" t="s">
+    <row r="110" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B110" s="2" t="s">
         <v>1958</v>
       </c>
-      <c r="C103" s="2" t="s">
+      <c r="C110" s="2" t="s">
         <v>1959</v>
       </c>
-      <c r="D103" s="2" t="s">
+      <c r="D110" s="2" t="s">
         <v>1960</v>
       </c>
-      <c r="E103" s="2" t="s">
+      <c r="E110" s="2" t="s">
         <v>1961</v>
       </c>
-      <c r="F103" s="2" t="s">
+      <c r="F110" s="2" t="s">
         <v>1962</v>
       </c>
-      <c r="G103" s="2" t="s">
+      <c r="G110" s="2" t="s">
         <v>1963</v>
       </c>
     </row>
-    <row r="104" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B104" s="2" t="s">
+    <row r="111" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B111" s="2" t="s">
         <v>1964</v>
       </c>
-      <c r="C104" s="2" t="s">
+      <c r="C111" s="2" t="s">
         <v>1965</v>
       </c>
-      <c r="D104" s="2" t="s">
+      <c r="D111" s="2" t="s">
         <v>1965</v>
       </c>
-      <c r="E104" s="2" t="s">
+      <c r="E111" s="2" t="s">
         <v>1966</v>
       </c>
-      <c r="F104" s="2" t="s">
+      <c r="F111" s="2" t="s">
         <v>1967</v>
       </c>
-      <c r="G104" s="2" t="s">
+      <c r="G111" s="2" t="s">
         <v>1968</v>
       </c>
     </row>
-    <row r="105" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B105" s="2" t="s">
+    <row r="112" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B112" s="2" t="s">
         <v>1969</v>
       </c>
-      <c r="C105" s="2" t="s">
+      <c r="C112" s="2" t="s">
         <v>1970</v>
       </c>
-      <c r="D105" s="2" t="s">
+      <c r="D112" s="2" t="s">
         <v>1971</v>
       </c>
-      <c r="E105" s="2" t="s">
+      <c r="E112" s="2" t="s">
         <v>1972</v>
       </c>
-      <c r="F105" s="2" t="s">
+      <c r="F112" s="2" t="s">
         <v>1973</v>
       </c>
-      <c r="G105" s="2" t="s">
+      <c r="G112" s="2" t="s">
         <v>1974</v>
       </c>
     </row>
-    <row r="106" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B106" s="2" t="s">
+    <row r="113" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B113" s="2" t="s">
         <v>1975</v>
       </c>
-      <c r="C106" s="2" t="s">
+      <c r="C113" s="2" t="s">
         <v>1976</v>
       </c>
-      <c r="D106" s="2" t="s">
+      <c r="D113" s="2" t="s">
         <v>1977</v>
       </c>
-      <c r="E106" s="2" t="s">
+      <c r="E113" s="2" t="s">
         <v>1978</v>
       </c>
-      <c r="F106" s="2" t="s">
+      <c r="F113" s="2" t="s">
         <v>1979</v>
       </c>
-      <c r="G106" s="2" t="s">
+      <c r="G113" s="2" t="s">
         <v>1980</v>
       </c>
     </row>
-    <row r="107" spans="2:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B107" s="2" t="s">
+    <row r="114" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="B114" s="2" t="s">
         <v>1981</v>
       </c>
-      <c r="C107" s="2" t="s">
+      <c r="C114" s="2" t="s">
         <v>1982</v>
       </c>
-      <c r="D107" s="2" t="s">
+      <c r="D114" s="2" t="s">
         <v>1983</v>
       </c>
-      <c r="E107" s="2" t="s">
+      <c r="E114" s="2" t="s">
         <v>1984</v>
       </c>
-      <c r="F107" s="2" t="s">
+      <c r="F114" s="2" t="s">
         <v>1985</v>
       </c>
-      <c r="G107" s="2" t="s">
+      <c r="G114" s="2" t="s">
         <v>1986</v>
       </c>
     </row>
-    <row r="111" spans="2:7" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="B111" s="3" t="s">
+    <row r="115" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15"/>
+    <row r="118" spans="2:7" ht="16" x14ac:dyDescent="0.15">
+      <c r="B118" s="3" t="s">
         <v>2037</v>
       </c>
     </row>
-    <row r="113" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B113" s="5" t="s">
+    <row r="120" spans="2:7" ht="13" x14ac:dyDescent="0.15">
+      <c r="B120" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C113" s="5" t="s">
+      <c r="C120" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="D113" s="5" t="s">
+      <c r="D120" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="E113" s="5" t="s">
+      <c r="E120" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="F113" s="5" t="s">
+      <c r="F120" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="G113" s="6" t="s">
+      <c r="G120" s="6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="114" spans="2:7" x14ac:dyDescent="0.2">
-      <c r="B114" s="7" t="s">
+    <row r="121" spans="2:7" ht="13" x14ac:dyDescent="0.15">
+      <c r="B121" s="7" t="s">
         <v>2038</v>
       </c>
-      <c r="C114" s="7" t="s">
+      <c r="C121" s="7" t="s">
         <v>2039</v>
       </c>
-      <c r="D114" s="7" t="s">
+      <c r="D121" s="7" t="s">
         <v>2043</v>
       </c>
-      <c r="E114" s="7" t="s">
+      <c r="E121" s="7" t="s">
         <v>2042</v>
       </c>
-      <c r="F114" s="7" t="s">
+      <c r="F121" s="7" t="s">
         <v>2041</v>
       </c>
-      <c r="G114" s="7" t="s">
+      <c r="G121" s="7" t="s">
         <v>2040</v>
       </c>
     </row>

</xml_diff>

<commit_message>
updated LinelistSpecs with temporary repos
</commit_message>
<xml_diff>
--- a/trads/designer_translations.xlsx
+++ b/trads/designer_translations.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/komlaviamevoin/Unsync-Working-Folders/outbreak-tools/trads/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Y:\trads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C13007D4-93A2-064E-B5E7-6D6CC6EF1936}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E928B431-3638-4FD6-8E7E-9D4FDA4B59AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="600" windowWidth="43800" windowHeight="29960" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="45315" windowHeight="24856" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LinelistTranslation" sheetId="1" r:id="rId1"/>
@@ -6256,7 +6256,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="9"/>
       <color rgb="FF000000"/>
@@ -6301,6 +6301,11 @@
       <name val="Helvetica"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+    </font>
   </fonts>
   <fills count="5">
     <fill>
@@ -6327,7 +6332,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="5">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -6375,11 +6380,22 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="4" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -6403,6 +6419,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7104,12 +7123,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="B2:G334"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="11.65" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="200" width="35.59765625" customWidth="1"/>
+    <col min="1" max="200" width="35.58203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="1" t="s">
         <v>0</v>
       </c>
@@ -7119,7 +7138,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -7127,7 +7146,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>2</v>
       </c>
@@ -7137,7 +7156,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -7145,7 +7164,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
@@ -7165,7 +7184,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="2" t="s">
         <v>9</v>
       </c>
@@ -7185,7 +7204,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="8" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="2" t="s">
         <v>15</v>
       </c>
@@ -7205,7 +7224,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="2" t="s">
         <v>21</v>
       </c>
@@ -7225,7 +7244,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="2" t="s">
         <v>27</v>
       </c>
@@ -7245,7 +7264,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="11" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="2" t="s">
         <v>33</v>
       </c>
@@ -7265,7 +7284,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="12" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="2" t="s">
         <v>37</v>
       </c>
@@ -7285,7 +7304,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="13" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="2" t="s">
         <v>42</v>
       </c>
@@ -7305,7 +7324,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="2" t="s">
         <v>45</v>
       </c>
@@ -7325,7 +7344,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="15" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="2" t="s">
         <v>50</v>
       </c>
@@ -7345,7 +7364,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="16" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="2" t="s">
         <v>56</v>
       </c>
@@ -7365,7 +7384,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="3" t="s">
         <v>62</v>
       </c>
@@ -7375,7 +7394,7 @@
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
     </row>
-    <row r="20" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="2"/>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -7383,7 +7402,7 @@
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
     </row>
-    <row r="21" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="2" t="s">
         <v>3</v>
       </c>
@@ -7403,7 +7422,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="22" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="2" t="s">
         <v>2013</v>
       </c>
@@ -7423,7 +7442,7 @@
         <v>2018</v>
       </c>
     </row>
-    <row r="23" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="2" t="s">
         <v>2019</v>
       </c>
@@ -7443,7 +7462,7 @@
         <v>2021</v>
       </c>
     </row>
-    <row r="24" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="2" t="s">
         <v>63</v>
       </c>
@@ -7463,7 +7482,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="2" t="s">
         <v>67</v>
       </c>
@@ -7483,7 +7502,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="26" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="2" t="s">
         <v>73</v>
       </c>
@@ -7503,7 +7522,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B27" s="2" t="s">
         <v>79</v>
       </c>
@@ -7523,7 +7542,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="2" t="s">
         <v>85</v>
       </c>
@@ -7543,7 +7562,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="29" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="2" t="s">
         <v>91</v>
       </c>
@@ -7563,7 +7582,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="2" t="s">
         <v>97</v>
       </c>
@@ -7583,7 +7602,7 @@
         <v>102</v>
       </c>
     </row>
-    <row r="31" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B31" s="2" t="s">
         <v>103</v>
       </c>
@@ -7603,7 +7622,7 @@
         <v>104</v>
       </c>
     </row>
-    <row r="32" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B32" s="2" t="s">
         <v>108</v>
       </c>
@@ -7623,7 +7642,7 @@
         <v>109</v>
       </c>
     </row>
-    <row r="33" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B33" s="2" t="s">
         <v>113</v>
       </c>
@@ -7643,7 +7662,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="34" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="34" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B34" s="2" t="s">
         <v>118</v>
       </c>
@@ -7663,7 +7682,7 @@
         <v>119</v>
       </c>
     </row>
-    <row r="35" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="2" t="s">
         <v>123</v>
       </c>
@@ -7683,7 +7702,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="36" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="36" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B36" s="2" t="s">
         <v>129</v>
       </c>
@@ -7703,7 +7722,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="37" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="37" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B37" s="2" t="s">
         <v>135</v>
       </c>
@@ -7723,7 +7742,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="38" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="38" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B38" s="2" t="s">
         <v>140</v>
       </c>
@@ -7743,7 +7762,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="39" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="39" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B39" s="2" t="s">
         <v>145</v>
       </c>
@@ -7763,7 +7782,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="40" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="40" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B40" s="2" t="s">
         <v>150</v>
       </c>
@@ -7783,7 +7802,7 @@
         <v>155</v>
       </c>
     </row>
-    <row r="41" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="41" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B41" s="2" t="s">
         <v>156</v>
       </c>
@@ -7803,7 +7822,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="42" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="42" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B42" s="2" t="s">
         <v>161</v>
       </c>
@@ -7823,7 +7842,7 @@
         <v>165</v>
       </c>
     </row>
-    <row r="43" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="43" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B43" s="2" t="s">
         <v>166</v>
       </c>
@@ -7843,7 +7862,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="44" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="44" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B44" s="2" t="s">
         <v>172</v>
       </c>
@@ -7863,7 +7882,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="45" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="45" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B45" s="2" t="s">
         <v>178</v>
       </c>
@@ -7883,7 +7902,7 @@
         <v>179</v>
       </c>
     </row>
-    <row r="46" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="46" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B46" s="2" t="s">
         <v>183</v>
       </c>
@@ -7903,7 +7922,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="47" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="47" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B47" s="2" t="s">
         <v>189</v>
       </c>
@@ -7923,7 +7942,7 @@
         <v>194</v>
       </c>
     </row>
-    <row r="48" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="48" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B48" s="2" t="s">
         <v>195</v>
       </c>
@@ -7943,7 +7962,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="49" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="49" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B49" s="2" t="s">
         <v>201</v>
       </c>
@@ -7963,7 +7982,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="50" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="50" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B50" s="2" t="s">
         <v>207</v>
       </c>
@@ -7983,7 +8002,7 @@
         <v>208</v>
       </c>
     </row>
-    <row r="51" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="51" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B51" s="2" t="s">
         <v>212</v>
       </c>
@@ -8003,7 +8022,7 @@
         <v>213</v>
       </c>
     </row>
-    <row r="52" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="52" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B52" s="2" t="s">
         <v>217</v>
       </c>
@@ -8023,7 +8042,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="53" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="53" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B53" s="2" t="s">
         <v>222</v>
       </c>
@@ -8043,7 +8062,7 @@
         <v>227</v>
       </c>
     </row>
-    <row r="54" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="54" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B54" s="2" t="s">
         <v>228</v>
       </c>
@@ -8063,7 +8082,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="55" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="55" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B55" s="2" t="s">
         <v>230</v>
       </c>
@@ -8083,7 +8102,7 @@
         <v>231</v>
       </c>
     </row>
-    <row r="56" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="56" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B56" s="2" t="s">
         <v>235</v>
       </c>
@@ -8103,7 +8122,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="57" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="57" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B57" s="2" t="s">
         <v>240</v>
       </c>
@@ -8123,7 +8142,7 @@
         <v>241</v>
       </c>
     </row>
-    <row r="58" spans="2:7" ht="39" x14ac:dyDescent="0.15">
+    <row r="58" spans="2:7" ht="34.9" x14ac:dyDescent="0.35">
       <c r="B58" s="2" t="s">
         <v>245</v>
       </c>
@@ -8143,7 +8162,7 @@
         <v>246</v>
       </c>
     </row>
-    <row r="59" spans="2:7" ht="51" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="59" spans="2:7" ht="51" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B59" s="4" t="s">
         <v>2007</v>
       </c>
@@ -8163,7 +8182,7 @@
         <v>2012</v>
       </c>
     </row>
-    <row r="60" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="60" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B60" s="2" t="s">
         <v>250</v>
       </c>
@@ -8183,7 +8202,7 @@
         <v>255</v>
       </c>
     </row>
-    <row r="61" spans="2:7" ht="52" x14ac:dyDescent="0.15">
+    <row r="61" spans="2:7" ht="46.5" x14ac:dyDescent="0.35">
       <c r="B61" s="2" t="s">
         <v>256</v>
       </c>
@@ -8203,7 +8222,7 @@
         <v>261</v>
       </c>
     </row>
-    <row r="62" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="62" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B62" s="2" t="s">
         <v>262</v>
       </c>
@@ -8223,7 +8242,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="63" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="63" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B63" s="2" t="s">
         <v>268</v>
       </c>
@@ -8243,7 +8262,7 @@
         <v>273</v>
       </c>
     </row>
-    <row r="64" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="64" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B64" s="2" t="s">
         <v>274</v>
       </c>
@@ -8263,7 +8282,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="65" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="65" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B65" s="2" t="s">
         <v>279</v>
       </c>
@@ -8283,7 +8302,7 @@
         <v>284</v>
       </c>
     </row>
-    <row r="66" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="66" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B66" s="2" t="s">
         <v>285</v>
       </c>
@@ -8301,7 +8320,7 @@
       </c>
       <c r="G66" s="2"/>
     </row>
-    <row r="67" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="67" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B67" s="2" t="s">
         <v>289</v>
       </c>
@@ -8321,7 +8340,7 @@
         <v>290</v>
       </c>
     </row>
-    <row r="68" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="68" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B68" s="2" t="s">
         <v>294</v>
       </c>
@@ -8341,7 +8360,7 @@
         <v>299</v>
       </c>
     </row>
-    <row r="69" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="69" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B69" s="2" t="s">
         <v>300</v>
       </c>
@@ -8361,7 +8380,7 @@
         <v>301</v>
       </c>
     </row>
-    <row r="70" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="70" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B70" s="2" t="s">
         <v>305</v>
       </c>
@@ -8381,7 +8400,7 @@
         <v>306</v>
       </c>
     </row>
-    <row r="71" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="71" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B71" s="2" t="s">
         <v>310</v>
       </c>
@@ -8401,7 +8420,7 @@
         <v>315</v>
       </c>
     </row>
-    <row r="72" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="72" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B72" s="2" t="s">
         <v>316</v>
       </c>
@@ -8421,7 +8440,7 @@
         <v>321</v>
       </c>
     </row>
-    <row r="73" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="73" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B73" s="2" t="s">
         <v>322</v>
       </c>
@@ -8441,7 +8460,7 @@
         <v>327</v>
       </c>
     </row>
-    <row r="74" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="74" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B74" s="2" t="s">
         <v>328</v>
       </c>
@@ -8461,7 +8480,7 @@
         <v>333</v>
       </c>
     </row>
-    <row r="75" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="75" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B75" s="2" t="s">
         <v>334</v>
       </c>
@@ -8481,7 +8500,7 @@
         <v>339</v>
       </c>
     </row>
-    <row r="76" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="76" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B76" s="2" t="s">
         <v>340</v>
       </c>
@@ -8501,7 +8520,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="77" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="77" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B77" s="2" t="s">
         <v>346</v>
       </c>
@@ -8521,7 +8540,7 @@
         <v>351</v>
       </c>
     </row>
-    <row r="78" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="78" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B78" s="2" t="s">
         <v>352</v>
       </c>
@@ -8541,7 +8560,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="79" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="79" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B79" s="2" t="s">
         <v>357</v>
       </c>
@@ -8561,7 +8580,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="80" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="80" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B80" s="2" t="s">
         <v>362</v>
       </c>
@@ -8581,7 +8600,7 @@
         <v>367</v>
       </c>
     </row>
-    <row r="81" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="81" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B81" s="2" t="s">
         <v>368</v>
       </c>
@@ -8601,7 +8620,7 @@
         <v>369</v>
       </c>
     </row>
-    <row r="82" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="82" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B82" s="2" t="s">
         <v>373</v>
       </c>
@@ -8621,7 +8640,7 @@
         <v>374</v>
       </c>
     </row>
-    <row r="83" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="83" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B83" s="2" t="s">
         <v>378</v>
       </c>
@@ -8641,7 +8660,7 @@
         <v>383</v>
       </c>
     </row>
-    <row r="84" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="84" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B84" s="2" t="s">
         <v>384</v>
       </c>
@@ -8661,7 +8680,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="85" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="85" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B85" s="2" t="s">
         <v>389</v>
       </c>
@@ -8681,7 +8700,7 @@
         <v>393</v>
       </c>
     </row>
-    <row r="86" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="86" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B86" s="2" t="s">
         <v>394</v>
       </c>
@@ -8701,7 +8720,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="87" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="87" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B87" s="2" t="s">
         <v>399</v>
       </c>
@@ -8721,7 +8740,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="88" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="88" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B88" s="2" t="s">
         <v>405</v>
       </c>
@@ -8741,7 +8760,7 @@
         <v>406</v>
       </c>
     </row>
-    <row r="89" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="89" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B89" s="2" t="s">
         <v>410</v>
       </c>
@@ -8761,7 +8780,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="90" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="90" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B90" s="2" t="s">
         <v>416</v>
       </c>
@@ -8781,7 +8800,7 @@
         <v>417</v>
       </c>
     </row>
-    <row r="91" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="91" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B91" s="2" t="s">
         <v>421</v>
       </c>
@@ -8801,7 +8820,7 @@
         <v>426</v>
       </c>
     </row>
-    <row r="92" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="92" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B92" s="2" t="s">
         <v>427</v>
       </c>
@@ -8821,7 +8840,7 @@
         <v>432</v>
       </c>
     </row>
-    <row r="93" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="93" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B93" s="2" t="s">
         <v>433</v>
       </c>
@@ -8841,7 +8860,7 @@
         <v>434</v>
       </c>
     </row>
-    <row r="94" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="94" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B94" s="2" t="s">
         <v>438</v>
       </c>
@@ -8861,7 +8880,7 @@
         <v>443</v>
       </c>
     </row>
-    <row r="95" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="95" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B95" s="2" t="s">
         <v>444</v>
       </c>
@@ -8881,7 +8900,7 @@
         <v>445</v>
       </c>
     </row>
-    <row r="96" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="96" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B96" s="2" t="s">
         <v>449</v>
       </c>
@@ -8901,7 +8920,7 @@
         <v>452</v>
       </c>
     </row>
-    <row r="97" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="97" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B97" s="2" t="s">
         <v>453</v>
       </c>
@@ -8921,7 +8940,7 @@
         <v>458</v>
       </c>
     </row>
-    <row r="98" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="98" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B98" s="2" t="s">
         <v>459</v>
       </c>
@@ -8941,7 +8960,7 @@
         <v>464</v>
       </c>
     </row>
-    <row r="99" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="99" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B99" s="2" t="s">
         <v>465</v>
       </c>
@@ -8961,7 +8980,7 @@
         <v>470</v>
       </c>
     </row>
-    <row r="100" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="100" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B100" s="2" t="s">
         <v>471</v>
       </c>
@@ -8981,7 +9000,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="101" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="101" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B101" s="2" t="s">
         <v>477</v>
       </c>
@@ -9001,7 +9020,7 @@
         <v>482</v>
       </c>
     </row>
-    <row r="102" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="102" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B102" s="2" t="s">
         <v>483</v>
       </c>
@@ -9021,7 +9040,7 @@
         <v>488</v>
       </c>
     </row>
-    <row r="103" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="103" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B103" s="2" t="s">
         <v>489</v>
       </c>
@@ -9041,7 +9060,7 @@
         <v>493</v>
       </c>
     </row>
-    <row r="104" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="104" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B104" s="2" t="s">
         <v>494</v>
       </c>
@@ -9061,7 +9080,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="105" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="105" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B105" s="2" t="s">
         <v>500</v>
       </c>
@@ -9081,7 +9100,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="106" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="106" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B106" s="2" t="s">
         <v>506</v>
       </c>
@@ -9101,7 +9120,7 @@
         <v>507</v>
       </c>
     </row>
-    <row r="107" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="107" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B107" s="2" t="s">
         <v>511</v>
       </c>
@@ -9121,7 +9140,7 @@
         <v>516</v>
       </c>
     </row>
-    <row r="108" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="108" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B108" s="2" t="s">
         <v>517</v>
       </c>
@@ -9141,7 +9160,7 @@
         <v>522</v>
       </c>
     </row>
-    <row r="109" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="109" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B109" s="2" t="s">
         <v>523</v>
       </c>
@@ -9161,7 +9180,7 @@
         <v>524</v>
       </c>
     </row>
-    <row r="110" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="110" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B110" s="2" t="s">
         <v>528</v>
       </c>
@@ -9181,7 +9200,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="111" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="111" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B111" s="2" t="s">
         <v>534</v>
       </c>
@@ -9201,7 +9220,7 @@
         <v>539</v>
       </c>
     </row>
-    <row r="112" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="112" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B112" s="2" t="s">
         <v>540</v>
       </c>
@@ -9221,7 +9240,7 @@
         <v>545</v>
       </c>
     </row>
-    <row r="113" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="113" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B113" s="2" t="s">
         <v>546</v>
       </c>
@@ -9241,7 +9260,7 @@
         <v>551</v>
       </c>
     </row>
-    <row r="114" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="114" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B114" s="2" t="s">
         <v>552</v>
       </c>
@@ -9261,7 +9280,7 @@
         <v>557</v>
       </c>
     </row>
-    <row r="115" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="115" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B115" s="2" t="s">
         <v>558</v>
       </c>
@@ -9281,7 +9300,7 @@
         <v>559</v>
       </c>
     </row>
-    <row r="116" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="116" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B116" s="2" t="s">
         <v>563</v>
       </c>
@@ -9301,7 +9320,7 @@
         <v>568</v>
       </c>
     </row>
-    <row r="117" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="117" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B117" s="2" t="s">
         <v>569</v>
       </c>
@@ -9321,7 +9340,7 @@
         <v>572</v>
       </c>
     </row>
-    <row r="118" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="118" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B118" s="2" t="s">
         <v>573</v>
       </c>
@@ -9341,7 +9360,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="119" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="119" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B119" s="2" t="s">
         <v>579</v>
       </c>
@@ -9361,7 +9380,7 @@
         <v>584</v>
       </c>
     </row>
-    <row r="120" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="120" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B120" s="2" t="s">
         <v>585</v>
       </c>
@@ -9381,7 +9400,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="121" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="121" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B121" s="2" t="s">
         <v>591</v>
       </c>
@@ -9401,7 +9420,7 @@
         <v>596</v>
       </c>
     </row>
-    <row r="122" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="122" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B122" s="2" t="s">
         <v>597</v>
       </c>
@@ -9421,7 +9440,7 @@
         <v>602</v>
       </c>
     </row>
-    <row r="123" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="123" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B123" s="2" t="s">
         <v>603</v>
       </c>
@@ -9441,7 +9460,7 @@
         <v>608</v>
       </c>
     </row>
-    <row r="124" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="124" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B124" s="2" t="s">
         <v>609</v>
       </c>
@@ -9461,7 +9480,7 @@
         <v>614</v>
       </c>
     </row>
-    <row r="125" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="125" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B125" s="2" t="s">
         <v>615</v>
       </c>
@@ -9481,7 +9500,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="126" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="126" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B126" s="2" t="s">
         <v>621</v>
       </c>
@@ -9501,7 +9520,7 @@
         <v>626</v>
       </c>
     </row>
-    <row r="127" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="127" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B127" s="2" t="s">
         <v>627</v>
       </c>
@@ -9521,7 +9540,7 @@
         <v>632</v>
       </c>
     </row>
-    <row r="128" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="128" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B128" s="2" t="s">
         <v>633</v>
       </c>
@@ -9541,7 +9560,7 @@
         <v>638</v>
       </c>
     </row>
-    <row r="129" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="129" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B129" s="2" t="s">
         <v>639</v>
       </c>
@@ -9561,7 +9580,7 @@
         <v>644</v>
       </c>
     </row>
-    <row r="130" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="130" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B130" s="2" t="s">
         <v>645</v>
       </c>
@@ -9581,7 +9600,7 @@
         <v>646</v>
       </c>
     </row>
-    <row r="131" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="131" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B131" s="2" t="s">
         <v>650</v>
       </c>
@@ -9601,7 +9620,7 @@
         <v>651</v>
       </c>
     </row>
-    <row r="132" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="132" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B132" s="2" t="s">
         <v>655</v>
       </c>
@@ -9621,7 +9640,7 @@
         <v>656</v>
       </c>
     </row>
-    <row r="133" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="133" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B133" s="2" t="s">
         <v>660</v>
       </c>
@@ -9641,7 +9660,7 @@
         <v>661</v>
       </c>
     </row>
-    <row r="134" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="134" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B134" s="2" t="s">
         <v>665</v>
       </c>
@@ -9661,7 +9680,7 @@
         <v>670</v>
       </c>
     </row>
-    <row r="135" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="135" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B135" s="2" t="s">
         <v>671</v>
       </c>
@@ -9681,7 +9700,7 @@
         <v>672</v>
       </c>
     </row>
-    <row r="136" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="136" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B136" s="2" t="s">
         <v>676</v>
       </c>
@@ -9701,7 +9720,7 @@
         <v>677</v>
       </c>
     </row>
-    <row r="137" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="137" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B137" s="2" t="s">
         <v>681</v>
       </c>
@@ -9721,7 +9740,7 @@
         <v>682</v>
       </c>
     </row>
-    <row r="138" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="138" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B138" s="2" t="s">
         <v>686</v>
       </c>
@@ -9741,7 +9760,7 @@
         <v>688</v>
       </c>
     </row>
-    <row r="139" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="139" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B139" s="2" t="s">
         <v>689</v>
       </c>
@@ -9761,7 +9780,7 @@
         <v>693</v>
       </c>
     </row>
-    <row r="140" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="140" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B140" s="2" t="s">
         <v>694</v>
       </c>
@@ -9781,7 +9800,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="141" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="141" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B141" s="2" t="s">
         <v>700</v>
       </c>
@@ -9801,7 +9820,7 @@
         <v>701</v>
       </c>
     </row>
-    <row r="142" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="142" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B142" s="2" t="s">
         <v>705</v>
       </c>
@@ -9819,7 +9838,7 @@
       </c>
       <c r="G142" s="2"/>
     </row>
-    <row r="143" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="143" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B143" s="2" t="s">
         <v>710</v>
       </c>
@@ -9839,7 +9858,7 @@
         <v>715</v>
       </c>
     </row>
-    <row r="144" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="144" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B144" s="2" t="s">
         <v>716</v>
       </c>
@@ -9859,7 +9878,7 @@
         <v>721</v>
       </c>
     </row>
-    <row r="145" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="145" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B145" s="2" t="s">
         <v>722</v>
       </c>
@@ -9879,7 +9898,7 @@
         <v>724</v>
       </c>
     </row>
-    <row r="146" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="146" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B146" s="2" t="s">
         <v>725</v>
       </c>
@@ -9899,7 +9918,7 @@
         <v>729</v>
       </c>
     </row>
-    <row r="147" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="147" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B147" s="2" t="s">
         <v>730</v>
       </c>
@@ -9919,7 +9938,7 @@
         <v>731</v>
       </c>
     </row>
-    <row r="148" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="148" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B148" s="2" t="s">
         <v>735</v>
       </c>
@@ -9939,7 +9958,7 @@
         <v>740</v>
       </c>
     </row>
-    <row r="149" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="149" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B149" s="2" t="s">
         <v>741</v>
       </c>
@@ -9957,7 +9976,7 @@
       </c>
       <c r="G149" s="2"/>
     </row>
-    <row r="150" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="150" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B150" s="2" t="s">
         <v>746</v>
       </c>
@@ -9977,7 +9996,7 @@
         <v>751</v>
       </c>
     </row>
-    <row r="151" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="151" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B151" s="2" t="s">
         <v>752</v>
       </c>
@@ -9997,7 +10016,7 @@
         <v>757</v>
       </c>
     </row>
-    <row r="152" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="152" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B152" s="2" t="s">
         <v>758</v>
       </c>
@@ -10017,7 +10036,7 @@
         <v>763</v>
       </c>
     </row>
-    <row r="153" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="153" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B153" s="2" t="s">
         <v>764</v>
       </c>
@@ -10037,7 +10056,7 @@
         <v>476</v>
       </c>
     </row>
-    <row r="154" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="154" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B154" s="2" t="s">
         <v>767</v>
       </c>
@@ -10057,7 +10076,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="155" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="155" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B155" s="2" t="s">
         <v>773</v>
       </c>
@@ -10077,7 +10096,7 @@
         <v>778</v>
       </c>
     </row>
-    <row r="156" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="156" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B156" s="2" t="s">
         <v>779</v>
       </c>
@@ -10097,7 +10116,7 @@
         <v>784</v>
       </c>
     </row>
-    <row r="157" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="157" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B157" s="2" t="s">
         <v>785</v>
       </c>
@@ -10117,7 +10136,7 @@
         <v>578</v>
       </c>
     </row>
-    <row r="158" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="158" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B158" s="2" t="s">
         <v>786</v>
       </c>
@@ -10137,7 +10156,7 @@
         <v>791</v>
       </c>
     </row>
-    <row r="159" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="159" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B159" s="2" t="s">
         <v>792</v>
       </c>
@@ -10157,7 +10176,7 @@
         <v>797</v>
       </c>
     </row>
-    <row r="160" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="160" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B160" s="2" t="s">
         <v>798</v>
       </c>
@@ -10177,7 +10196,7 @@
         <v>803</v>
       </c>
     </row>
-    <row r="161" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="161" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B161" s="2" t="s">
         <v>804</v>
       </c>
@@ -10197,7 +10216,7 @@
         <v>415</v>
       </c>
     </row>
-    <row r="162" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="162" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B162" s="2" t="s">
         <v>809</v>
       </c>
@@ -10217,7 +10236,7 @@
         <v>814</v>
       </c>
     </row>
-    <row r="163" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="163" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B163" s="2" t="s">
         <v>815</v>
       </c>
@@ -10237,7 +10256,7 @@
         <v>820</v>
       </c>
     </row>
-    <row r="164" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="164" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B164" s="2" t="s">
         <v>821</v>
       </c>
@@ -10257,7 +10276,7 @@
         <v>823</v>
       </c>
     </row>
-    <row r="165" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="165" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B165" s="2" t="s">
         <v>824</v>
       </c>
@@ -10277,7 +10296,7 @@
         <v>829</v>
       </c>
     </row>
-    <row r="166" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="166" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B166" s="2" t="s">
         <v>830</v>
       </c>
@@ -10297,7 +10316,7 @@
         <v>835</v>
       </c>
     </row>
-    <row r="167" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="167" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B167" s="2" t="s">
         <v>836</v>
       </c>
@@ -10317,7 +10336,7 @@
         <v>840</v>
       </c>
     </row>
-    <row r="168" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="168" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B168" s="2" t="s">
         <v>841</v>
       </c>
@@ -10337,7 +10356,7 @@
         <v>845</v>
       </c>
     </row>
-    <row r="169" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="169" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B169" s="2" t="s">
         <v>846</v>
       </c>
@@ -10357,7 +10376,7 @@
         <v>851</v>
       </c>
     </row>
-    <row r="170" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="170" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B170" s="2" t="s">
         <v>852</v>
       </c>
@@ -10377,7 +10396,7 @@
         <v>856</v>
       </c>
     </row>
-    <row r="171" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="171" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B171" s="2" t="s">
         <v>857</v>
       </c>
@@ -10397,7 +10416,7 @@
         <v>858</v>
       </c>
     </row>
-    <row r="172" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="172" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B172" s="2" t="s">
         <v>862</v>
       </c>
@@ -10417,7 +10436,7 @@
         <v>867</v>
       </c>
     </row>
-    <row r="173" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="173" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B173" s="2" t="s">
         <v>868</v>
       </c>
@@ -10437,7 +10456,7 @@
         <v>873</v>
       </c>
     </row>
-    <row r="174" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="174" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B174" s="2" t="s">
         <v>874</v>
       </c>
@@ -10457,7 +10476,7 @@
         <v>879</v>
       </c>
     </row>
-    <row r="175" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="175" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B175" s="2" t="s">
         <v>880</v>
       </c>
@@ -10477,7 +10496,7 @@
         <v>885</v>
       </c>
     </row>
-    <row r="176" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="176" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B176" s="2" t="s">
         <v>886</v>
       </c>
@@ -10497,7 +10516,7 @@
         <v>890</v>
       </c>
     </row>
-    <row r="177" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="177" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B177" s="2" t="s">
         <v>1991</v>
       </c>
@@ -10517,7 +10536,7 @@
         <v>1996</v>
       </c>
     </row>
-    <row r="178" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="178" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B178" s="4" t="s">
         <v>1997</v>
       </c>
@@ -10537,7 +10556,7 @@
         <v>2000</v>
       </c>
     </row>
-    <row r="181" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="181" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B181" s="3" t="s">
         <v>891</v>
       </c>
@@ -10547,7 +10566,7 @@
       <c r="F181" s="2"/>
       <c r="G181" s="2"/>
     </row>
-    <row r="182" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="182" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B182" s="2"/>
       <c r="C182" s="2"/>
       <c r="D182" s="2"/>
@@ -10555,7 +10574,7 @@
       <c r="F182" s="2"/>
       <c r="G182" s="2"/>
     </row>
-    <row r="183" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="183" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B183" s="2" t="s">
         <v>3</v>
       </c>
@@ -10575,7 +10594,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="184" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="184" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B184" s="2" t="s">
         <v>892</v>
       </c>
@@ -10595,7 +10614,7 @@
         <v>897</v>
       </c>
     </row>
-    <row r="185" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="185" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B185" s="2" t="s">
         <v>898</v>
       </c>
@@ -10615,7 +10634,7 @@
         <v>900</v>
       </c>
     </row>
-    <row r="186" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="186" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B186" s="2" t="s">
         <v>901</v>
       </c>
@@ -10635,7 +10654,7 @@
         <v>906</v>
       </c>
     </row>
-    <row r="187" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="187" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B187" s="2" t="s">
         <v>907</v>
       </c>
@@ -10655,7 +10674,7 @@
         <v>910</v>
       </c>
     </row>
-    <row r="188" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="188" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B188" s="2" t="s">
         <v>911</v>
       </c>
@@ -10675,7 +10694,7 @@
         <v>916</v>
       </c>
     </row>
-    <row r="189" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="189" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B189" s="2" t="s">
         <v>917</v>
       </c>
@@ -10695,7 +10714,7 @@
         <v>922</v>
       </c>
     </row>
-    <row r="190" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="190" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B190" s="2" t="s">
         <v>923</v>
       </c>
@@ -10715,7 +10734,7 @@
         <v>927</v>
       </c>
     </row>
-    <row r="191" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="191" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B191" s="2" t="s">
         <v>928</v>
       </c>
@@ -10735,7 +10754,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="192" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="192" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B192" s="2" t="s">
         <v>934</v>
       </c>
@@ -10755,7 +10774,7 @@
         <v>939</v>
       </c>
     </row>
-    <row r="193" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="193" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B193" s="2" t="s">
         <v>940</v>
       </c>
@@ -10775,7 +10794,7 @@
         <v>945</v>
       </c>
     </row>
-    <row r="194" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="194" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B194" s="2" t="s">
         <v>946</v>
       </c>
@@ -10795,7 +10814,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="195" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="195" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B195" s="2" t="s">
         <v>948</v>
       </c>
@@ -10815,7 +10834,7 @@
         <v>953</v>
       </c>
     </row>
-    <row r="196" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="196" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B196" s="2" t="s">
         <v>954</v>
       </c>
@@ -10835,7 +10854,7 @@
         <v>959</v>
       </c>
     </row>
-    <row r="197" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="197" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B197" s="2" t="s">
         <v>960</v>
       </c>
@@ -10855,7 +10874,7 @@
         <v>964</v>
       </c>
     </row>
-    <row r="198" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="198" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B198" s="2" t="s">
         <v>965</v>
       </c>
@@ -10875,7 +10894,7 @@
         <v>969</v>
       </c>
     </row>
-    <row r="199" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="199" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B199" s="2" t="s">
         <v>970</v>
       </c>
@@ -10895,7 +10914,7 @@
         <v>971</v>
       </c>
     </row>
-    <row r="200" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="200" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B200" s="2" t="s">
         <v>972</v>
       </c>
@@ -10915,7 +10934,7 @@
         <v>976</v>
       </c>
     </row>
-    <row r="201" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="201" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B201" s="2" t="s">
         <v>977</v>
       </c>
@@ -10935,7 +10954,7 @@
         <v>981</v>
       </c>
     </row>
-    <row r="202" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="202" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B202" s="2" t="s">
         <v>982</v>
       </c>
@@ -10955,7 +10974,7 @@
         <v>985</v>
       </c>
     </row>
-    <row r="203" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="203" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B203" s="2" t="s">
         <v>986</v>
       </c>
@@ -10975,7 +10994,7 @@
         <v>990</v>
       </c>
     </row>
-    <row r="204" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="204" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B204" s="2" t="s">
         <v>991</v>
       </c>
@@ -10995,7 +11014,7 @@
         <v>992</v>
       </c>
     </row>
-    <row r="205" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="205" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B205" s="2" t="s">
         <v>993</v>
       </c>
@@ -11015,7 +11034,7 @@
         <v>994</v>
       </c>
     </row>
-    <row r="206" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="206" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B206" s="2" t="s">
         <v>995</v>
       </c>
@@ -11035,7 +11054,7 @@
         <v>996</v>
       </c>
     </row>
-    <row r="207" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="207" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B207" s="2" t="s">
         <v>997</v>
       </c>
@@ -11055,7 +11074,7 @@
         <v>998</v>
       </c>
     </row>
-    <row r="208" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="208" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B208" s="2" t="s">
         <v>999</v>
       </c>
@@ -11075,7 +11094,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="209" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="209" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B209" s="2" t="s">
         <v>1004</v>
       </c>
@@ -11095,7 +11114,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="210" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="210" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B210" s="2" t="s">
         <v>1006</v>
       </c>
@@ -11115,7 +11134,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="211" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="211" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B211" s="2" t="s">
         <v>1007</v>
       </c>
@@ -11135,7 +11154,7 @@
         <v>1012</v>
       </c>
     </row>
-    <row r="212" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="212" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B212" s="2" t="s">
         <v>1013</v>
       </c>
@@ -11155,7 +11174,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="213" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="213" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B213" s="2" t="s">
         <v>1014</v>
       </c>
@@ -11175,7 +11194,7 @@
         <v>1019</v>
       </c>
     </row>
-    <row r="214" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="214" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B214" s="2" t="s">
         <v>1020</v>
       </c>
@@ -11195,7 +11214,7 @@
         <v>1024</v>
       </c>
     </row>
-    <row r="215" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="215" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B215" s="2" t="s">
         <v>1025</v>
       </c>
@@ -11215,7 +11234,7 @@
         <v>1030</v>
       </c>
     </row>
-    <row r="216" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="216" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B216" s="2" t="s">
         <v>1031</v>
       </c>
@@ -11235,7 +11254,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="217" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="217" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B217" s="2" t="s">
         <v>1032</v>
       </c>
@@ -11255,7 +11274,7 @@
         <v>1037</v>
       </c>
     </row>
-    <row r="218" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="218" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B218" s="2" t="s">
         <v>1038</v>
       </c>
@@ -11275,7 +11294,7 @@
         <v>1043</v>
       </c>
     </row>
-    <row r="219" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="219" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B219" s="2" t="s">
         <v>1044</v>
       </c>
@@ -11295,7 +11314,7 @@
         <v>1049</v>
       </c>
     </row>
-    <row r="220" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="220" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B220" s="2" t="s">
         <v>1050</v>
       </c>
@@ -11315,7 +11334,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="221" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="221" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B221" s="2" t="s">
         <v>1051</v>
       </c>
@@ -11335,7 +11354,7 @@
         <v>1056</v>
       </c>
     </row>
-    <row r="222" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="222" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B222" s="2" t="s">
         <v>1057</v>
       </c>
@@ -11355,7 +11374,7 @@
         <v>1062</v>
       </c>
     </row>
-    <row r="223" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="223" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B223" s="2" t="s">
         <v>1063</v>
       </c>
@@ -11375,7 +11394,7 @@
         <v>1068</v>
       </c>
     </row>
-    <row r="224" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="224" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B224" s="2" t="s">
         <v>1069</v>
       </c>
@@ -11395,7 +11414,7 @@
         <v>1074</v>
       </c>
     </row>
-    <row r="225" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="225" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B225" s="2" t="s">
         <v>1075</v>
       </c>
@@ -11415,7 +11434,7 @@
         <v>933</v>
       </c>
     </row>
-    <row r="226" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="226" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B226" s="2" t="s">
         <v>1076</v>
       </c>
@@ -11435,7 +11454,7 @@
         <v>1080</v>
       </c>
     </row>
-    <row r="227" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="227" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B227" s="2" t="s">
         <v>1081</v>
       </c>
@@ -11455,7 +11474,7 @@
         <v>1086</v>
       </c>
     </row>
-    <row r="228" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="228" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B228" s="2" t="s">
         <v>1087</v>
       </c>
@@ -11475,7 +11494,7 @@
         <v>505</v>
       </c>
     </row>
-    <row r="229" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="229" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B229" s="2" t="s">
         <v>1091</v>
       </c>
@@ -11495,7 +11514,7 @@
         <v>1096</v>
       </c>
     </row>
-    <row r="230" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="230" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B230" s="2" t="s">
         <v>1097</v>
       </c>
@@ -11515,7 +11534,7 @@
         <v>939</v>
       </c>
     </row>
-    <row r="231" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="231" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B231" s="2" t="s">
         <v>1098</v>
       </c>
@@ -11535,7 +11554,7 @@
         <v>945</v>
       </c>
     </row>
-    <row r="232" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="232" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B232" s="2" t="s">
         <v>1102</v>
       </c>
@@ -11555,7 +11574,7 @@
         <v>1107</v>
       </c>
     </row>
-    <row r="233" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="233" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B233" s="2" t="s">
         <v>1108</v>
       </c>
@@ -11575,7 +11594,7 @@
         <v>1989</v>
       </c>
     </row>
-    <row r="234" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="234" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B234" s="2" t="s">
         <v>1109</v>
       </c>
@@ -11595,7 +11614,7 @@
         <v>1110</v>
       </c>
     </row>
-    <row r="235" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="235" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B235" s="2" t="s">
         <v>1113</v>
       </c>
@@ -11615,7 +11634,7 @@
         <v>590</v>
       </c>
     </row>
-    <row r="236" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="236" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B236" s="2" t="s">
         <v>1114</v>
       </c>
@@ -11635,7 +11654,7 @@
         <v>1118</v>
       </c>
     </row>
-    <row r="237" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="237" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B237" s="2" t="s">
         <v>1119</v>
       </c>
@@ -11655,7 +11674,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="238" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="238" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B238" s="2" t="s">
         <v>1120</v>
       </c>
@@ -11675,7 +11694,7 @@
         <v>1125</v>
       </c>
     </row>
-    <row r="239" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="239" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B239" s="2" t="s">
         <v>1126</v>
       </c>
@@ -11695,7 +11714,7 @@
         <v>1131</v>
       </c>
     </row>
-    <row r="240" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="240" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B240" s="2" t="s">
         <v>1132</v>
       </c>
@@ -11715,7 +11734,7 @@
         <v>1131</v>
       </c>
     </row>
-    <row r="241" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="241" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B241" s="2" t="s">
         <v>1133</v>
       </c>
@@ -11735,7 +11754,7 @@
         <v>1138</v>
       </c>
     </row>
-    <row r="242" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="242" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B242" s="2" t="s">
         <v>1139</v>
       </c>
@@ -11755,7 +11774,7 @@
         <v>1141</v>
       </c>
     </row>
-    <row r="243" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="243" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B243" s="2" t="s">
         <v>1142</v>
       </c>
@@ -11775,7 +11794,7 @@
         <v>1141</v>
       </c>
     </row>
-    <row r="244" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="244" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B244" s="2" t="s">
         <v>1143</v>
       </c>
@@ -11795,7 +11814,7 @@
         <v>1145</v>
       </c>
     </row>
-    <row r="245" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="245" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B245" s="2" t="s">
         <v>1146</v>
       </c>
@@ -11815,7 +11834,7 @@
         <v>1145</v>
       </c>
     </row>
-    <row r="246" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="246" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B246" s="2" t="s">
         <v>1147</v>
       </c>
@@ -11835,7 +11854,7 @@
         <v>1149</v>
       </c>
     </row>
-    <row r="247" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="247" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B247" s="2" t="s">
         <v>1150</v>
       </c>
@@ -11855,7 +11874,7 @@
         <v>1149</v>
       </c>
     </row>
-    <row r="248" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="248" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B248" s="2" t="s">
         <v>1151</v>
       </c>
@@ -11875,7 +11894,7 @@
         <v>1153</v>
       </c>
     </row>
-    <row r="249" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="249" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B249" s="2" t="s">
         <v>1154</v>
       </c>
@@ -11895,7 +11914,7 @@
         <v>1153</v>
       </c>
     </row>
-    <row r="250" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="250" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B250" s="2" t="s">
         <v>1155</v>
       </c>
@@ -11915,7 +11934,7 @@
         <v>1160</v>
       </c>
     </row>
-    <row r="251" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="251" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B251" s="2" t="s">
         <v>1161</v>
       </c>
@@ -11935,7 +11954,7 @@
         <v>699</v>
       </c>
     </row>
-    <row r="252" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="252" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B252" s="2" t="s">
         <v>1164</v>
       </c>
@@ -11955,7 +11974,7 @@
         <v>1169</v>
       </c>
     </row>
-    <row r="253" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="253" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B253" s="2" t="s">
         <v>1170</v>
       </c>
@@ -11975,7 +11994,7 @@
         <v>1175</v>
       </c>
     </row>
-    <row r="254" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="254" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B254" s="2" t="s">
         <v>1176</v>
       </c>
@@ -11995,7 +12014,7 @@
         <v>1181</v>
       </c>
     </row>
-    <row r="255" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="255" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B255" s="2" t="s">
         <v>1182</v>
       </c>
@@ -12015,7 +12034,7 @@
         <v>1185</v>
       </c>
     </row>
-    <row r="256" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="256" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B256" s="2" t="s">
         <v>1186</v>
       </c>
@@ -12035,7 +12054,7 @@
         <v>1191</v>
       </c>
     </row>
-    <row r="257" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="257" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B257" s="2" t="s">
         <v>1192</v>
       </c>
@@ -12055,7 +12074,7 @@
         <v>1197</v>
       </c>
     </row>
-    <row r="258" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="258" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B258" s="2" t="s">
         <v>1198</v>
       </c>
@@ -12075,7 +12094,7 @@
         <v>1197</v>
       </c>
     </row>
-    <row r="259" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="259" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B259" s="2" t="s">
         <v>1199</v>
       </c>
@@ -12095,7 +12114,7 @@
         <v>1204</v>
       </c>
     </row>
-    <row r="260" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="260" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B260" s="2" t="s">
         <v>1205</v>
       </c>
@@ -12115,7 +12134,7 @@
         <v>1185</v>
       </c>
     </row>
-    <row r="261" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="261" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B261" s="2" t="s">
         <v>1206</v>
       </c>
@@ -12135,7 +12154,7 @@
         <v>1185</v>
       </c>
     </row>
-    <row r="262" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="262" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B262" s="2" t="s">
         <v>1207</v>
       </c>
@@ -12155,7 +12174,7 @@
         <v>1212</v>
       </c>
     </row>
-    <row r="263" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="263" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B263" s="2" t="s">
         <v>1213</v>
       </c>
@@ -12175,7 +12194,7 @@
         <v>1218</v>
       </c>
     </row>
-    <row r="264" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="264" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B264" s="2" t="s">
         <v>1219</v>
       </c>
@@ -12195,7 +12214,7 @@
         <v>1224</v>
       </c>
     </row>
-    <row r="265" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="265" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B265" s="2" t="s">
         <v>1225</v>
       </c>
@@ -12215,7 +12234,7 @@
         <v>1230</v>
       </c>
     </row>
-    <row r="266" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="266" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B266" s="2" t="s">
         <v>1231</v>
       </c>
@@ -12235,7 +12254,7 @@
         <v>1235</v>
       </c>
     </row>
-    <row r="267" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="267" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B267" s="2" t="s">
         <v>1236</v>
       </c>
@@ -12255,7 +12274,7 @@
         <v>1240</v>
       </c>
     </row>
-    <row r="268" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="268" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B268" s="2" t="s">
         <v>1241</v>
       </c>
@@ -12275,7 +12294,7 @@
         <v>1246</v>
       </c>
     </row>
-    <row r="269" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="269" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B269" s="2" t="s">
         <v>1247</v>
       </c>
@@ -12295,7 +12314,7 @@
         <v>1246</v>
       </c>
     </row>
-    <row r="270" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="270" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B270" s="2" t="s">
         <v>1248</v>
       </c>
@@ -12315,7 +12334,7 @@
         <v>1246</v>
       </c>
     </row>
-    <row r="271" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="271" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B271" s="2" t="s">
         <v>1249</v>
       </c>
@@ -12335,7 +12354,7 @@
         <v>1246</v>
       </c>
     </row>
-    <row r="272" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="272" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B272" s="2" t="s">
         <v>1250</v>
       </c>
@@ -12355,7 +12374,7 @@
         <v>1255</v>
       </c>
     </row>
-    <row r="273" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="273" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B273" s="2" t="s">
         <v>1256</v>
       </c>
@@ -12375,7 +12394,7 @@
         <v>1235</v>
       </c>
     </row>
-    <row r="274" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="274" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B274" s="2" t="s">
         <v>1257</v>
       </c>
@@ -12395,7 +12414,7 @@
         <v>1240</v>
       </c>
     </row>
-    <row r="275" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="275" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B275" s="2" t="s">
         <v>1258</v>
       </c>
@@ -12415,7 +12434,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="276" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="276" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B276" s="2" t="s">
         <v>1259</v>
       </c>
@@ -12435,7 +12454,7 @@
         <v>1264</v>
       </c>
     </row>
-    <row r="277" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="277" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B277" s="2" t="s">
         <v>1265</v>
       </c>
@@ -12455,7 +12474,7 @@
         <v>1270</v>
       </c>
     </row>
-    <row r="278" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="278" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B278" s="2" t="s">
         <v>1271</v>
       </c>
@@ -12475,7 +12494,7 @@
         <v>772</v>
       </c>
     </row>
-    <row r="279" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="279" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B279" s="2" t="s">
         <v>1272</v>
       </c>
@@ -12495,7 +12514,7 @@
         <v>1277</v>
       </c>
     </row>
-    <row r="280" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="280" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B280" s="2" t="s">
         <v>1278</v>
       </c>
@@ -12515,7 +12534,7 @@
         <v>1283</v>
       </c>
     </row>
-    <row r="281" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="281" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B281" s="2" t="s">
         <v>1284</v>
       </c>
@@ -12535,7 +12554,7 @@
         <v>1287</v>
       </c>
     </row>
-    <row r="282" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="282" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B282" s="2" t="s">
         <v>1288</v>
       </c>
@@ -12555,7 +12574,7 @@
         <v>1292</v>
       </c>
     </row>
-    <row r="283" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="283" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B283" s="2" t="s">
         <v>1293</v>
       </c>
@@ -12575,7 +12594,7 @@
         <v>1298</v>
       </c>
     </row>
-    <row r="284" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="284" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B284" s="2" t="s">
         <v>1299</v>
       </c>
@@ -12595,7 +12614,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="285" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="285" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B285" s="2" t="s">
         <v>1305</v>
       </c>
@@ -12615,7 +12634,7 @@
         <v>1310</v>
       </c>
     </row>
-    <row r="286" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="286" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B286" s="2" t="s">
         <v>1311</v>
       </c>
@@ -12635,7 +12654,7 @@
         <v>1316</v>
       </c>
     </row>
-    <row r="287" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="287" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B287" s="2" t="s">
         <v>1317</v>
       </c>
@@ -12655,7 +12674,7 @@
         <v>1316</v>
       </c>
     </row>
-    <row r="288" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="288" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B288" s="2" t="s">
         <v>1318</v>
       </c>
@@ -12675,7 +12694,7 @@
         <v>1323</v>
       </c>
     </row>
-    <row r="289" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="289" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B289" s="2" t="s">
         <v>1324</v>
       </c>
@@ -12695,7 +12714,7 @@
         <v>1323</v>
       </c>
     </row>
-    <row r="290" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="290" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B290" s="2" t="s">
         <v>1325</v>
       </c>
@@ -12715,7 +12734,7 @@
         <v>1329</v>
       </c>
     </row>
-    <row r="291" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="291" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B291" s="2" t="s">
         <v>1330</v>
       </c>
@@ -12735,7 +12754,7 @@
         <v>1329</v>
       </c>
     </row>
-    <row r="292" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="292" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B292" s="2"/>
       <c r="C292" s="2"/>
       <c r="D292" s="2"/>
@@ -12743,7 +12762,7 @@
       <c r="F292" s="2"/>
       <c r="G292" s="2"/>
     </row>
-    <row r="293" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="293" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B293" s="2"/>
       <c r="C293" s="2"/>
       <c r="D293" s="2"/>
@@ -12751,7 +12770,7 @@
       <c r="F293" s="2"/>
       <c r="G293" s="2"/>
     </row>
-    <row r="294" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="294" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B294" s="3" t="s">
         <v>1331</v>
       </c>
@@ -12761,7 +12780,7 @@
       <c r="F294" s="2"/>
       <c r="G294" s="2"/>
     </row>
-    <row r="295" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="295" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B295" s="2"/>
       <c r="C295" s="2"/>
       <c r="D295" s="2"/>
@@ -12769,7 +12788,7 @@
       <c r="F295" s="2"/>
       <c r="G295" s="2"/>
     </row>
-    <row r="296" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="296" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B296" s="2" t="s">
         <v>3</v>
       </c>
@@ -12789,7 +12808,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="297" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="297" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B297" s="2" t="s">
         <v>1332</v>
       </c>
@@ -12809,7 +12828,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="298" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="298" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B298" s="2" t="s">
         <v>1334</v>
       </c>
@@ -12829,7 +12848,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="299" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="299" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B299" s="2" t="s">
         <v>1337</v>
       </c>
@@ -12849,7 +12868,7 @@
         <v>1342</v>
       </c>
     </row>
-    <row r="300" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="300" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B300" s="2" t="s">
         <v>1343</v>
       </c>
@@ -12869,7 +12888,7 @@
         <v>1346</v>
       </c>
     </row>
-    <row r="301" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="301" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B301" s="2" t="s">
         <v>1347</v>
       </c>
@@ -12889,7 +12908,7 @@
         <v>1349</v>
       </c>
     </row>
-    <row r="302" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="302" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B302" s="2" t="s">
         <v>1350</v>
       </c>
@@ -12909,7 +12928,7 @@
         <v>1355</v>
       </c>
     </row>
-    <row r="303" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="303" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B303" s="2" t="s">
         <v>1356</v>
       </c>
@@ -12929,7 +12948,7 @@
         <v>1361</v>
       </c>
     </row>
-    <row r="304" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="304" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B304" s="2" t="s">
         <v>1362</v>
       </c>
@@ -12949,7 +12968,7 @@
         <v>1367</v>
       </c>
     </row>
-    <row r="305" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="305" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B305" s="2" t="s">
         <v>1368</v>
       </c>
@@ -12969,7 +12988,7 @@
         <v>2006</v>
       </c>
     </row>
-    <row r="306" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="306" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B306" s="2" t="s">
         <v>1369</v>
       </c>
@@ -12989,7 +13008,7 @@
         <v>1118</v>
       </c>
     </row>
-    <row r="307" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="307" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B307" s="2" t="s">
         <v>1372</v>
       </c>
@@ -13009,7 +13028,7 @@
         <v>1376</v>
       </c>
     </row>
-    <row r="308" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="308" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B308" s="2" t="s">
         <v>1377</v>
       </c>
@@ -13029,7 +13048,7 @@
         <v>1382</v>
       </c>
     </row>
-    <row r="309" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="309" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B309" s="2" t="s">
         <v>1383</v>
       </c>
@@ -13049,7 +13068,7 @@
         <v>1388</v>
       </c>
     </row>
-    <row r="310" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="310" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B310" s="2" t="s">
         <v>1389</v>
       </c>
@@ -13069,7 +13088,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="311" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="311" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B311" s="2" t="s">
         <v>1390</v>
       </c>
@@ -13089,7 +13108,7 @@
         <v>1019</v>
       </c>
     </row>
-    <row r="312" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="312" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B312" s="2" t="s">
         <v>1391</v>
       </c>
@@ -13109,7 +13128,7 @@
         <v>1393</v>
       </c>
     </row>
-    <row r="313" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="313" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B313" s="2" t="s">
         <v>1394</v>
       </c>
@@ -13129,7 +13148,7 @@
         <v>1398</v>
       </c>
     </row>
-    <row r="314" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="314" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B314" s="2" t="s">
         <v>1399</v>
       </c>
@@ -13149,7 +13168,7 @@
         <v>1404</v>
       </c>
     </row>
-    <row r="315" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="315" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B315" s="2" t="s">
         <v>1405</v>
       </c>
@@ -13169,7 +13188,7 @@
         <v>1410</v>
       </c>
     </row>
-    <row r="316" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="316" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B316" s="2" t="s">
         <v>1411</v>
       </c>
@@ -13189,7 +13208,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="317" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="317" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B317" s="2" t="s">
         <v>1412</v>
       </c>
@@ -13209,7 +13228,7 @@
         <v>1417</v>
       </c>
     </row>
-    <row r="318" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="318" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B318" s="2" t="s">
         <v>1418</v>
       </c>
@@ -13229,7 +13248,7 @@
         <v>1423</v>
       </c>
     </row>
-    <row r="319" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="319" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B319" s="2" t="s">
         <v>1424</v>
       </c>
@@ -13249,7 +13268,7 @@
         <v>1429</v>
       </c>
     </row>
-    <row r="320" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="320" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B320" s="2" t="s">
         <v>1430</v>
       </c>
@@ -13269,7 +13288,7 @@
         <v>1435</v>
       </c>
     </row>
-    <row r="321" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="321" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B321" s="2" t="s">
         <v>1436</v>
       </c>
@@ -13289,7 +13308,7 @@
         <v>1441</v>
       </c>
     </row>
-    <row r="322" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="322" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B322" s="2" t="s">
         <v>1442</v>
       </c>
@@ -13309,7 +13328,7 @@
         <v>1447</v>
       </c>
     </row>
-    <row r="323" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="323" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B323" s="2" t="s">
         <v>1448</v>
       </c>
@@ -13329,7 +13348,7 @@
         <v>1451</v>
       </c>
     </row>
-    <row r="324" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="324" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B324" s="2" t="s">
         <v>1452</v>
       </c>
@@ -13349,7 +13368,7 @@
         <v>1457</v>
       </c>
     </row>
-    <row r="325" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="325" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B325" s="2" t="s">
         <v>1458</v>
       </c>
@@ -13369,7 +13388,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="326" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="326" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B326" s="2" t="s">
         <v>1459</v>
       </c>
@@ -13389,7 +13408,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="327" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="327" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B327" s="2" t="s">
         <v>1460</v>
       </c>
@@ -13409,7 +13428,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="328" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="328" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B328" s="2" t="s">
         <v>1461</v>
       </c>
@@ -13429,7 +13448,7 @@
         <v>533</v>
       </c>
     </row>
-    <row r="329" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="329" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B329" s="2" t="s">
         <v>1463</v>
       </c>
@@ -13449,7 +13468,7 @@
         <v>1468</v>
       </c>
     </row>
-    <row r="330" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="330" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B330" s="2" t="s">
         <v>1469</v>
       </c>
@@ -13469,7 +13488,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="331" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="331" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B331" s="2" t="s">
         <v>1470</v>
       </c>
@@ -13489,7 +13508,7 @@
         <v>1475</v>
       </c>
     </row>
-    <row r="332" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="332" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B332" s="2" t="s">
         <v>1476</v>
       </c>
@@ -13509,7 +13528,7 @@
         <v>1480</v>
       </c>
     </row>
-    <row r="333" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="333" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B333" s="2" t="s">
         <v>1481</v>
       </c>
@@ -13529,7 +13548,7 @@
         <v>1482</v>
       </c>
     </row>
-    <row r="334" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="334" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B334" s="2" t="s">
         <v>1483</v>
       </c>
@@ -13565,12 +13584,12 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr codeName="Sheet2"/>
   <dimension ref="B2:G121"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="12" defaultRowHeight="12" x14ac:dyDescent="0.15"/>
+  <sheetFormatPr defaultColWidth="12" defaultRowHeight="11.65" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="200" width="35.59765625" customWidth="1"/>
+    <col min="1" max="200" width="35.58203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="2" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B2" s="1" t="s">
         <v>1</v>
       </c>
@@ -13580,7 +13599,7 @@
       <c r="F2" s="2"/>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="3" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B3" s="2"/>
       <c r="C3" s="2"/>
       <c r="D3" s="2"/>
@@ -13588,7 +13607,7 @@
       <c r="F3" s="2"/>
       <c r="G3" s="2"/>
     </row>
-    <row r="4" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="4" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B4" s="3" t="s">
         <v>1489</v>
       </c>
@@ -13598,7 +13617,7 @@
       <c r="F4" s="2"/>
       <c r="G4" s="2"/>
     </row>
-    <row r="5" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="5" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B5" s="2"/>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -13606,7 +13625,7 @@
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
     </row>
-    <row r="6" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="6" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B6" s="2" t="s">
         <v>3</v>
       </c>
@@ -13626,7 +13645,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="7" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B7" s="2" t="s">
         <v>1827</v>
       </c>
@@ -13646,7 +13665,7 @@
         <v>1107</v>
       </c>
     </row>
-    <row r="8" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="8" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B8" s="2" t="s">
         <v>1579</v>
       </c>
@@ -13666,7 +13685,7 @@
         <v>1584</v>
       </c>
     </row>
-    <row r="9" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="9" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B9" s="2" t="s">
         <v>1781</v>
       </c>
@@ -13686,7 +13705,7 @@
         <v>1786</v>
       </c>
     </row>
-    <row r="10" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="10" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B10" s="2" t="s">
         <v>1598</v>
       </c>
@@ -13706,7 +13725,7 @@
         <v>1603</v>
       </c>
     </row>
-    <row r="11" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="11" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B11" s="2" t="s">
         <v>1495</v>
       </c>
@@ -13726,7 +13745,7 @@
         <v>1500</v>
       </c>
     </row>
-    <row r="12" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="12" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B12" s="2" t="s">
         <v>1536</v>
       </c>
@@ -13746,7 +13765,7 @@
         <v>1541</v>
       </c>
     </row>
-    <row r="13" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="13" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B13" s="2" t="s">
         <v>1639</v>
       </c>
@@ -13766,7 +13785,7 @@
         <v>1643</v>
       </c>
     </row>
-    <row r="14" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="14" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B14" s="2" t="s">
         <v>1654</v>
       </c>
@@ -13786,7 +13805,7 @@
         <v>1659</v>
       </c>
     </row>
-    <row r="15" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="15" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B15" s="2" t="s">
         <v>1775</v>
       </c>
@@ -13806,7 +13825,7 @@
         <v>1780</v>
       </c>
     </row>
-    <row r="16" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="16" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B16" s="2" t="s">
         <v>1665</v>
       </c>
@@ -13826,7 +13845,7 @@
         <v>1666</v>
       </c>
     </row>
-    <row r="17" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="17" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B17" s="2" t="s">
         <v>1627</v>
       </c>
@@ -13846,7 +13865,7 @@
         <v>1632</v>
       </c>
     </row>
-    <row r="18" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="18" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B18" s="2" t="s">
         <v>1787</v>
       </c>
@@ -13866,7 +13885,7 @@
         <v>1791</v>
       </c>
     </row>
-    <row r="19" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="19" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B19" s="2" t="s">
         <v>1792</v>
       </c>
@@ -13886,7 +13905,7 @@
         <v>1797</v>
       </c>
     </row>
-    <row r="20" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="20" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B20" s="2" t="s">
         <v>1519</v>
       </c>
@@ -13906,7 +13925,7 @@
         <v>1524</v>
       </c>
     </row>
-    <row r="21" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="21" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B21" s="2" t="s">
         <v>1501</v>
       </c>
@@ -13926,7 +13945,7 @@
         <v>1506</v>
       </c>
     </row>
-    <row r="22" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="22" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B22" s="2" t="s">
         <v>1741</v>
       </c>
@@ -13946,7 +13965,7 @@
         <v>1742</v>
       </c>
     </row>
-    <row r="23" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="23" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B23" s="2" t="s">
         <v>1490</v>
       </c>
@@ -13966,7 +13985,7 @@
         <v>1491</v>
       </c>
     </row>
-    <row r="24" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="24" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B24" s="2" t="s">
         <v>1682</v>
       </c>
@@ -13986,7 +14005,7 @@
         <v>1687</v>
       </c>
     </row>
-    <row r="25" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="25" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B25" s="2" t="s">
         <v>274</v>
       </c>
@@ -14006,7 +14025,7 @@
         <v>1561</v>
       </c>
     </row>
-    <row r="26" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="26" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B26" s="2" t="s">
         <v>1591</v>
       </c>
@@ -14026,7 +14045,7 @@
         <v>1561</v>
       </c>
     </row>
-    <row r="27" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="27" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B27" s="2" t="s">
         <v>1568</v>
       </c>
@@ -14046,7 +14065,7 @@
         <v>1573</v>
       </c>
     </row>
-    <row r="28" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="28" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B28" s="2" t="s">
         <v>1548</v>
       </c>
@@ -14066,7 +14085,7 @@
         <v>1553</v>
       </c>
     </row>
-    <row r="29" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="29" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B29" s="2" t="s">
         <v>399</v>
       </c>
@@ -14086,7 +14105,7 @@
         <v>1578</v>
       </c>
     </row>
-    <row r="30" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="30" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B30" s="2" t="s">
         <v>1729</v>
       </c>
@@ -14106,7 +14125,7 @@
         <v>1734</v>
       </c>
     </row>
-    <row r="31" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="31" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B31" s="2" t="s">
         <v>1585</v>
       </c>
@@ -14126,7 +14145,7 @@
         <v>1590</v>
       </c>
     </row>
-    <row r="32" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="32" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B32" s="2" t="s">
         <v>1735</v>
       </c>
@@ -14146,7 +14165,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="33" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="33" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B33" s="2" t="s">
         <v>1763</v>
       </c>
@@ -14166,7 +14185,7 @@
         <v>1768</v>
       </c>
     </row>
-    <row r="34" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="34" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B34" s="2" t="s">
         <v>1821</v>
       </c>
@@ -14186,7 +14205,7 @@
         <v>1826</v>
       </c>
     </row>
-    <row r="35" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="35" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B35" s="2" t="s">
         <v>1798</v>
       </c>
@@ -14206,7 +14225,7 @@
         <v>1803</v>
       </c>
     </row>
-    <row r="36" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="36" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B36" s="2" t="s">
         <v>1804</v>
       </c>
@@ -14226,7 +14245,7 @@
         <v>1808</v>
       </c>
     </row>
-    <row r="37" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="37" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B37" s="2" t="s">
         <v>1815</v>
       </c>
@@ -14246,7 +14265,7 @@
         <v>1820</v>
       </c>
     </row>
-    <row r="38" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="38" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B38" s="2" t="s">
         <v>1700</v>
       </c>
@@ -14266,7 +14285,7 @@
         <v>1705</v>
       </c>
     </row>
-    <row r="39" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="39" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B39" s="2" t="s">
         <v>1828</v>
       </c>
@@ -14286,7 +14305,7 @@
         <v>1829</v>
       </c>
     </row>
-    <row r="40" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="40" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B40" s="4" t="s">
         <v>2024</v>
       </c>
@@ -14306,7 +14325,7 @@
         <v>2029</v>
       </c>
     </row>
-    <row r="41" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="41" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B41" s="2" t="s">
         <v>1836</v>
       </c>
@@ -14326,7 +14345,7 @@
         <v>1841</v>
       </c>
     </row>
-    <row r="42" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="42" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B42" s="2" t="s">
         <v>1513</v>
       </c>
@@ -14346,7 +14365,7 @@
         <v>1518</v>
       </c>
     </row>
-    <row r="43" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="43" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B43" s="2" t="s">
         <v>1830</v>
       </c>
@@ -14366,7 +14385,7 @@
         <v>1835</v>
       </c>
     </row>
-    <row r="44" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="44" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B44" s="2" t="s">
         <v>1621</v>
       </c>
@@ -14386,7 +14405,7 @@
         <v>1626</v>
       </c>
     </row>
-    <row r="45" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="45" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B45" s="2" t="s">
         <v>1649</v>
       </c>
@@ -14406,7 +14425,7 @@
         <v>1650</v>
       </c>
     </row>
-    <row r="46" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="46" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B46" s="2" t="s">
         <v>1809</v>
       </c>
@@ -14426,7 +14445,7 @@
         <v>1814</v>
       </c>
     </row>
-    <row r="47" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="47" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B47" s="2" t="s">
         <v>1644</v>
       </c>
@@ -14446,7 +14465,7 @@
         <v>1645</v>
       </c>
     </row>
-    <row r="48" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="48" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B48" s="2" t="s">
         <v>1736</v>
       </c>
@@ -14466,7 +14485,7 @@
         <v>1737</v>
       </c>
     </row>
-    <row r="49" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="49" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B49" s="2" t="s">
         <v>1745</v>
       </c>
@@ -14486,7 +14505,7 @@
         <v>1750</v>
       </c>
     </row>
-    <row r="50" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="50" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B50" s="2" t="s">
         <v>1615</v>
       </c>
@@ -14506,7 +14525,7 @@
         <v>1620</v>
       </c>
     </row>
-    <row r="51" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="51" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B51" s="2" t="s">
         <v>558</v>
       </c>
@@ -14526,7 +14545,7 @@
         <v>1614</v>
       </c>
     </row>
-    <row r="52" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="52" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B52" s="2" t="s">
         <v>1507</v>
       </c>
@@ -14546,7 +14565,7 @@
         <v>1512</v>
       </c>
     </row>
-    <row r="53" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="53" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B53" s="2" t="s">
         <v>1525</v>
       </c>
@@ -14566,7 +14585,7 @@
         <v>1530</v>
       </c>
     </row>
-    <row r="54" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="54" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B54" s="2" t="s">
         <v>1670</v>
       </c>
@@ -14586,7 +14605,7 @@
         <v>1675</v>
       </c>
     </row>
-    <row r="55" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="55" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B55" s="2" t="s">
         <v>1562</v>
       </c>
@@ -14606,7 +14625,7 @@
         <v>1567</v>
       </c>
     </row>
-    <row r="56" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="56" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B56" s="2" t="s">
         <v>1676</v>
       </c>
@@ -14626,7 +14645,7 @@
         <v>1681</v>
       </c>
     </row>
-    <row r="57" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="57" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B57" s="2" t="s">
         <v>1688</v>
       </c>
@@ -14646,7 +14665,7 @@
         <v>1693</v>
       </c>
     </row>
-    <row r="58" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="58" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B58" s="2" t="s">
         <v>1694</v>
       </c>
@@ -14666,7 +14685,7 @@
         <v>1699</v>
       </c>
     </row>
-    <row r="59" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="59" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B59" s="2" t="s">
         <v>1706</v>
       </c>
@@ -14686,7 +14705,7 @@
         <v>1711</v>
       </c>
     </row>
-    <row r="60" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="60" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B60" s="2" t="s">
         <v>1712</v>
       </c>
@@ -14706,7 +14725,7 @@
         <v>1717</v>
       </c>
     </row>
-    <row r="61" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="61" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B61" s="2" t="s">
         <v>1718</v>
       </c>
@@ -14726,7 +14745,7 @@
         <v>1723</v>
       </c>
     </row>
-    <row r="62" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="62" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B62" s="2" t="s">
         <v>1542</v>
       </c>
@@ -14746,7 +14765,7 @@
         <v>1547</v>
       </c>
     </row>
-    <row r="63" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="63" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B63" s="2" t="s">
         <v>1592</v>
       </c>
@@ -14766,7 +14785,7 @@
         <v>1597</v>
       </c>
     </row>
-    <row r="64" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="64" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B64" s="2" t="s">
         <v>1531</v>
       </c>
@@ -14786,7 +14805,7 @@
         <v>1532</v>
       </c>
     </row>
-    <row r="65" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="65" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B65" s="2" t="s">
         <v>1604</v>
       </c>
@@ -14806,7 +14825,7 @@
         <v>1609</v>
       </c>
     </row>
-    <row r="66" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="66" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B66" s="2" t="s">
         <v>1724</v>
       </c>
@@ -14826,7 +14845,7 @@
         <v>1725</v>
       </c>
     </row>
-    <row r="67" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="67" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B67" s="2" t="s">
         <v>1660</v>
       </c>
@@ -14846,7 +14865,7 @@
         <v>1661</v>
       </c>
     </row>
-    <row r="68" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="68" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B68" s="2" t="s">
         <v>1751</v>
       </c>
@@ -14866,7 +14885,7 @@
         <v>1756</v>
       </c>
     </row>
-    <row r="69" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="69" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B69" s="2" t="s">
         <v>1757</v>
       </c>
@@ -14886,7 +14905,7 @@
         <v>1762</v>
       </c>
     </row>
-    <row r="70" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="70" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B70" s="2" t="s">
         <v>1633</v>
       </c>
@@ -14906,7 +14925,7 @@
         <v>1638</v>
       </c>
     </row>
-    <row r="71" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="71" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B71" s="2" t="s">
         <v>1554</v>
       </c>
@@ -14926,7 +14945,7 @@
         <v>1559</v>
       </c>
     </row>
-    <row r="72" spans="2:7" ht="39" x14ac:dyDescent="0.15">
+    <row r="72" spans="2:7" ht="34.9" x14ac:dyDescent="0.35">
       <c r="B72" s="2" t="s">
         <v>1769</v>
       </c>
@@ -14946,7 +14965,7 @@
         <v>1774</v>
       </c>
     </row>
-    <row r="73" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="73" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B73" s="4" t="s">
         <v>2045</v>
       </c>
@@ -14966,7 +14985,7 @@
         <v>2048</v>
       </c>
     </row>
-    <row r="74" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="74" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B74" s="4" t="s">
         <v>2051</v>
       </c>
@@ -14986,7 +15005,7 @@
         <v>2062</v>
       </c>
     </row>
-    <row r="75" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="75" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B75" s="4" t="s">
         <v>2052</v>
       </c>
@@ -15006,7 +15025,7 @@
         <v>2063</v>
       </c>
     </row>
-    <row r="76" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="76" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B76" s="4" t="s">
         <v>2055</v>
       </c>
@@ -15026,7 +15045,7 @@
         <v>2061</v>
       </c>
     </row>
-    <row r="77" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="77" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B77" s="4" t="s">
         <v>2058</v>
       </c>
@@ -15046,7 +15065,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="78" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="78" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B78" s="8" t="s">
         <v>2066</v>
       </c>
@@ -15066,7 +15085,7 @@
         <v>1820</v>
       </c>
     </row>
-    <row r="79" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="79" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B79" s="8" t="s">
         <v>2067</v>
       </c>
@@ -15086,7 +15105,7 @@
         <v>2071</v>
       </c>
     </row>
-    <row r="80" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="80" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
       <c r="D80" s="2"/>
@@ -15094,7 +15113,7 @@
       <c r="F80" s="2"/>
       <c r="G80" s="2"/>
     </row>
-    <row r="81" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="81" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B81" s="3" t="s">
         <v>1842</v>
       </c>
@@ -15104,7 +15123,7 @@
       <c r="F81" s="2"/>
       <c r="G81" s="2"/>
     </row>
-    <row r="82" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="82" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B82" s="2"/>
       <c r="C82" s="2"/>
       <c r="D82" s="2"/>
@@ -15112,7 +15131,7 @@
       <c r="F82" s="2"/>
       <c r="G82" s="2"/>
     </row>
-    <row r="83" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="83" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B83" s="2" t="s">
         <v>3</v>
       </c>
@@ -15132,7 +15151,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="84" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="84" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B84" s="2" t="s">
         <v>1843</v>
       </c>
@@ -15152,7 +15171,7 @@
         <v>1848</v>
       </c>
     </row>
-    <row r="85" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="85" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B85" s="2" t="s">
         <v>1849</v>
       </c>
@@ -15172,7 +15191,7 @@
         <v>1853</v>
       </c>
     </row>
-    <row r="86" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="86" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B86" s="2" t="s">
         <v>1854</v>
       </c>
@@ -15192,7 +15211,7 @@
         <v>1859</v>
       </c>
     </row>
-    <row r="87" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="87" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B87" s="2" t="s">
         <v>1860</v>
       </c>
@@ -15212,7 +15231,7 @@
         <v>1865</v>
       </c>
     </row>
-    <row r="88" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="88" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B88" s="2" t="s">
         <v>1866</v>
       </c>
@@ -15232,7 +15251,7 @@
         <v>1871</v>
       </c>
     </row>
-    <row r="89" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="89" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B89" s="2" t="s">
         <v>1872</v>
       </c>
@@ -15252,7 +15271,7 @@
         <v>1877</v>
       </c>
     </row>
-    <row r="90" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="90" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B90" s="2" t="s">
         <v>1878</v>
       </c>
@@ -15272,7 +15291,7 @@
         <v>1883</v>
       </c>
     </row>
-    <row r="91" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="91" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B91" s="2" t="s">
         <v>1884</v>
       </c>
@@ -15292,7 +15311,7 @@
         <v>1889</v>
       </c>
     </row>
-    <row r="92" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="92" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B92" s="2" t="s">
         <v>1890</v>
       </c>
@@ -15312,7 +15331,7 @@
         <v>1895</v>
       </c>
     </row>
-    <row r="93" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="93" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B93" s="2" t="s">
         <v>1896</v>
       </c>
@@ -15332,7 +15351,7 @@
         <v>1841</v>
       </c>
     </row>
-    <row r="94" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="94" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B94" s="2" t="s">
         <v>1900</v>
       </c>
@@ -15352,7 +15371,7 @@
         <v>1905</v>
       </c>
     </row>
-    <row r="95" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="95" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B95" s="2" t="s">
         <v>1906</v>
       </c>
@@ -15372,7 +15391,7 @@
         <v>1911</v>
       </c>
     </row>
-    <row r="96" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="96" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B96" s="2" t="s">
         <v>1912</v>
       </c>
@@ -15392,35 +15411,34 @@
         <v>1916</v>
       </c>
     </row>
-    <row r="97" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="97" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B97" s="2" t="s">
         <v>2031</v>
       </c>
       <c r="C97" s="2" t="s">
-        <v>2032</v>
+        <v>2033</v>
       </c>
       <c r="D97" s="2" t="s">
-        <v>2033</v>
+        <v>2034</v>
       </c>
       <c r="E97" s="2" t="s">
-        <v>2034</v>
+        <v>2036</v>
       </c>
       <c r="F97" s="2" t="s">
         <v>2035</v>
       </c>
-      <c r="G97" s="2" t="s">
-        <v>2036</v>
-      </c>
-    </row>
-    <row r="98" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="G97" s="9" t="s">
+        <v>2032</v>
+      </c>
+    </row>
+    <row r="98" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
       <c r="D98" s="2"/>
-      <c r="E98" s="2"/>
       <c r="F98" s="2"/>
       <c r="G98" s="2"/>
     </row>
-    <row r="99" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="99" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B99" s="3" t="s">
         <v>1917</v>
       </c>
@@ -15430,7 +15448,7 @@
       <c r="F99" s="2"/>
       <c r="G99" s="2"/>
     </row>
-    <row r="100" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="100" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
       <c r="D100" s="2"/>
@@ -15438,7 +15456,7 @@
       <c r="F100" s="2"/>
       <c r="G100" s="2"/>
     </row>
-    <row r="101" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="101" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B101" s="2" t="s">
         <v>3</v>
       </c>
@@ -15458,7 +15476,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="102" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="102" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B102" s="2" t="s">
         <v>1918</v>
       </c>
@@ -15478,7 +15496,7 @@
         <v>1080</v>
       </c>
     </row>
-    <row r="103" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="103" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B103" s="2" t="s">
         <v>1919</v>
       </c>
@@ -15498,7 +15516,7 @@
         <v>1924</v>
       </c>
     </row>
-    <row r="104" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="104" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B104" s="2" t="s">
         <v>1925</v>
       </c>
@@ -15518,7 +15536,7 @@
         <v>1930</v>
       </c>
     </row>
-    <row r="105" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="105" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B105" s="2" t="s">
         <v>1931</v>
       </c>
@@ -15538,7 +15556,7 @@
         <v>1936</v>
       </c>
     </row>
-    <row r="106" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="106" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B106" s="2" t="s">
         <v>1937</v>
       </c>
@@ -15558,7 +15576,7 @@
         <v>1942</v>
       </c>
     </row>
-    <row r="107" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="107" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B107" s="2" t="s">
         <v>1943</v>
       </c>
@@ -15578,7 +15596,7 @@
         <v>1948</v>
       </c>
     </row>
-    <row r="108" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="108" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B108" s="2" t="s">
         <v>1949</v>
       </c>
@@ -15598,7 +15616,7 @@
         <v>1953</v>
       </c>
     </row>
-    <row r="109" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="109" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B109" s="2" t="s">
         <v>50</v>
       </c>
@@ -15618,7 +15636,7 @@
         <v>1957</v>
       </c>
     </row>
-    <row r="110" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="110" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B110" s="2" t="s">
         <v>1958</v>
       </c>
@@ -15638,7 +15656,7 @@
         <v>1963</v>
       </c>
     </row>
-    <row r="111" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="111" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B111" s="2" t="s">
         <v>1964</v>
       </c>
@@ -15658,7 +15676,7 @@
         <v>1968</v>
       </c>
     </row>
-    <row r="112" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="112" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B112" s="2" t="s">
         <v>1969</v>
       </c>
@@ -15678,7 +15696,7 @@
         <v>1974</v>
       </c>
     </row>
-    <row r="113" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="113" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B113" s="2" t="s">
         <v>1975</v>
       </c>
@@ -15698,7 +15716,7 @@
         <v>1980</v>
       </c>
     </row>
-    <row r="114" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15">
+    <row r="114" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35">
       <c r="B114" s="2" t="s">
         <v>1981</v>
       </c>
@@ -15718,13 +15736,13 @@
         <v>1986</v>
       </c>
     </row>
-    <row r="115" spans="2:7" ht="25" customHeight="1" x14ac:dyDescent="0.15"/>
-    <row r="118" spans="2:7" ht="16" x14ac:dyDescent="0.15">
+    <row r="115" spans="2:7" ht="25.05" customHeight="1" x14ac:dyDescent="0.35"/>
+    <row r="118" spans="2:7" ht="15.75" x14ac:dyDescent="0.35">
       <c r="B118" s="3" t="s">
         <v>2037</v>
       </c>
     </row>
-    <row r="120" spans="2:7" ht="13" x14ac:dyDescent="0.15">
+    <row r="120" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B120" s="5" t="s">
         <v>3</v>
       </c>
@@ -15744,7 +15762,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="121" spans="2:7" ht="13" x14ac:dyDescent="0.15">
+    <row r="121" spans="2:7" x14ac:dyDescent="0.35">
       <c r="B121" s="7" t="s">
         <v>2038</v>
       </c>
@@ -15766,12 +15784,12 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
   <tableParts count="4">
-    <tablePart r:id="rId1"/>
     <tablePart r:id="rId2"/>
     <tablePart r:id="rId3"/>
     <tablePart r:id="rId4"/>
+    <tablePart r:id="rId5"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>